<commit_message>
feat(timelines): add activity timelines page, fix catalogs, remove Mail.ru OAuth
- Add new GET /api/v1/ingest/users/timeline endpoint with hourly activity aggregation
- Create TimelinesPage with hierarchical user→groups→apps→sites view
- Gray bars for activity, red bars for activity with video recording
- Fix catalogs crash (TypeError: length) - backend returns array, not wrapper object
- Remove all Mail.ru OAuth code from auth-service and web-dashboard (keep Yandex)
- Replace vite.svg favicon with branded Kadero favicon.png
- Fix sidebar spacing between menu items and submenu
- Add "Таймлайны" to sidebar under "Аналитика" section

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracker.xlsx
+++ b/docs/tracker.xlsx
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I145"/>
+  <dimension ref="A1:I160"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="15" min="1" max="1"/>
@@ -2054,7 +2054,7 @@
       </c>
       <c r="F34" s="18" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Cancelled</t>
         </is>
       </c>
       <c r="G34" s="19" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="I34" s="18" t="inlineStr">
         <is>
-          <t>07.03.2026</t>
+          <t>09.03.2026</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="F35" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Cancelled</t>
         </is>
       </c>
       <c r="G35" s="19" t="inlineStr">
@@ -2116,7 +2116,7 @@
       </c>
       <c r="I35" s="18" t="inlineStr">
         <is>
-          <t>07.03.2026</t>
+          <t>09.03.2026</t>
         </is>
       </c>
     </row>
@@ -2289,7 +2289,7 @@
       </c>
       <c r="F39" s="24" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Cancelled</t>
         </is>
       </c>
       <c r="G39" s="25" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="I39" s="24" t="inlineStr">
         <is>
-          <t>07.03.2026</t>
+          <t>09.03.2026</t>
         </is>
       </c>
     </row>
@@ -7224,7 +7224,7 @@
       </c>
       <c r="F144" s="18" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G144" s="19" t="inlineStr">
@@ -7271,20 +7271,725 @@
       </c>
       <c r="F145" s="18" t="inlineStr">
         <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G145" s="19" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="H145" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+      <c r="I145" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="20" customHeight="1" s="15">
+      <c r="A146" s="18" t="inlineStr">
+        <is>
+          <t>T-141</t>
+        </is>
+      </c>
+      <c r="B146" s="18" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C146" s="19" t="inlineStr">
+        <is>
+          <t>Agent Lifecycle: функциональное тестирование heartbeat, status-log, device-settings</t>
+        </is>
+      </c>
+      <c r="D146" s="19" t="inlineStr">
+        <is>
+          <t>Тестирование полного цикла жизни агента: heartbeat с новыми статусами (starting, configuring, awaiting_user, idle, stopped, recording, online, error, offline), Status-Log API, device settings defaults, tenant isolation</t>
+        </is>
+      </c>
+      <c r="E146" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F146" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G146" s="19" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="H146" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+      <c r="I146" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="20" customHeight="1" s="15">
+      <c r="A147" s="18" t="inlineStr">
+        <is>
+          <t>T-142</t>
+        </is>
+      </c>
+      <c r="B147" s="18" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C147" s="19" t="inlineStr">
+        <is>
+          <t>Backend: endpoint GET /users/timeline в UserActivityController</t>
+        </is>
+      </c>
+      <c r="D147" s="19" t="inlineStr">
+        <is>
+          <t>Новый endpoint GET /api/v1/ingest/users/timeline?date=...&amp;timezone=... для почасовой агрегации активности пользователей с иерархией групп приложений/сайтов. Permission: RECORDINGS:READ. Спецификация: docs/timelines-spec.md раздел 4.1</t>
+        </is>
+      </c>
+      <c r="E147" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F147" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G147" s="19" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="H147" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+      <c r="I147" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="20" customHeight="1" s="15">
+      <c r="A148" s="18" t="inlineStr">
+        <is>
+          <t>T-143</t>
+        </is>
+      </c>
+      <c r="B148" s="18" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C148" s="19" t="inlineStr">
+        <is>
+          <t>Backend: TimelineService с SQL-агрегацией и кэшем групп</t>
+        </is>
+      </c>
+      <c r="D148" s="19" t="inlineStr">
+        <is>
+          <t>Сервис с 3 SQL-запросами (focus_intervals агрегация по часам, recording_sessions за день, device_user_sessions маппинг). In-memory сборка иерархии user-&gt;hour-&gt;group-&gt;app/domain. Кэш app_group_items для tenant (TTL 5мин). Спецификация: docs/timelines-spec.md раздел 4.2-4.3</t>
+        </is>
+      </c>
+      <c r="E148" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F148" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G148" s="19" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="H148" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+      <c r="I148" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="20" customHeight="1" s="15">
+      <c r="A149" s="18" t="inlineStr">
+        <is>
+          <t>T-144</t>
+        </is>
+      </c>
+      <c r="B149" s="18" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C149" s="19" t="inlineStr">
+        <is>
+          <t>Backend: DTO TimelineResponse + вложенные модели</t>
+        </is>
+      </c>
+      <c r="D149" s="19" t="inlineStr">
+        <is>
+          <t>Java DTO: TimelineResponse, TimelineUser, TimelineHour, TimelineAppGroup, TimelineApp, TimelineSiteGroup, TimelineSite. Спецификация: docs/timelines-spec.md раздел 4.1</t>
+        </is>
+      </c>
+      <c r="E149" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F149" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G149" s="19" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="H149" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+      <c r="I149" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="20" customHeight="1" s="15">
+      <c r="A150" s="18" t="inlineStr">
+        <is>
+          <t>T-145</t>
+        </is>
+      </c>
+      <c r="B150" s="18" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C150" s="19" t="inlineStr">
+        <is>
+          <t>Удалить Mail.ru OAuth из auth-service (backend)</t>
+        </is>
+      </c>
+      <c r="D150" s="19" t="inlineStr">
+        <is>
+          <t>Удалить: MailruOAuthConfig.java, MailruOAuthClient.java, MailruOAuthClientTest.java (файлы). В OAuthService.java: удалить mailruClient, mailruOAuthConfig, PROVIDER_MAILRU, getMailruAuthorizationUrl(), handleMailruCallback(). В OAuthController.java: удалить mailruOAuthConfig, endpoints /mailru и /mailru/callback, ветку mailru в processOAuthCallback(). В SecurityConfig.java: удалить 2 строки permitAll. В application.yml: удалить блок mailru. Спецификация: docs/timelines-spec.md раздел 9</t>
+        </is>
+      </c>
+      <c r="E150" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F150" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G150" s="19" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="H150" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+      <c r="I150" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="20" customHeight="1" s="15">
+      <c r="A151" s="18" t="inlineStr">
+        <is>
+          <t>T-146</t>
+        </is>
+      </c>
+      <c r="B151" s="18" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C151" s="19" t="inlineStr">
+        <is>
+          <t>Frontend: страница TimelinesPage + компоненты таймлайна</t>
+        </is>
+      </c>
+      <c r="D151" s="19" t="inlineStr">
+        <is>
+          <t>Новая страница TimelinesPage.tsx. Компоненты: TimelineTable, TimelineRow (Level 1: пользователь), TimelineBar (серая/красная колбаска), TimelineAppGroupRow (Level 2), TimelineAppRow (Level 3), TimelineSiteGroupRow (Level 3 для браузеров), TimelineSiteRow (Level 4), TimelineDatePicker. Спецификация: docs/timelines-spec.md раздел 6</t>
+        </is>
+      </c>
+      <c r="E151" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F151" s="18" t="inlineStr">
+        <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="G145" s="19" t="inlineStr">
+      <c r="G151" s="19" t="inlineStr">
         <is>
           <t>Frontend</t>
         </is>
       </c>
-      <c r="H145" s="18" t="inlineStr">
+      <c r="H151" s="18" t="inlineStr">
         <is>
           <t>09.03.2026</t>
         </is>
       </c>
-      <c r="I145" s="18" t="inlineStr">
+      <c r="I151" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="20" customHeight="1" s="15">
+      <c r="A152" s="18" t="inlineStr">
+        <is>
+          <t>T-147</t>
+        </is>
+      </c>
+      <c r="B152" s="18" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C152" s="19" t="inlineStr">
+        <is>
+          <t>Frontend: типы Timeline* + API функция getTimeline()</t>
+        </is>
+      </c>
+      <c r="D152" s="19" t="inlineStr">
+        <is>
+          <t>TypeScript типы в types/user-activity.ts: TimelineResponse, TimelineUser, TimelineHour, TimelineAppGroup, TimelineApp, TimelineSiteGroup, TimelineSite. Функция getTimeline() в api/user-activity.ts: GET /users/timeline?date=...&amp;timezone=... Спецификация: docs/timelines-spec.md раздел 4.1 и 6.5</t>
+        </is>
+      </c>
+      <c r="E152" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F152" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G152" s="19" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="H152" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+      <c r="I152" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="20" customHeight="1" s="15">
+      <c r="A153" s="18" t="inlineStr">
+        <is>
+          <t>T-148</t>
+        </is>
+      </c>
+      <c r="B153" s="18" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C153" s="19" t="inlineStr">
+        <is>
+          <t>Frontend: маршрут /archive/timelines + подпункт Sidebar</t>
+        </is>
+      </c>
+      <c r="D153" s="19" t="inlineStr">
+        <is>
+          <t>Добавить Route path=/archive/timelines element=TimelinesPage в App.tsx. Добавить NavItem 'Таймлайны' с href=/archive/timelines и icon=ClockIcon в archiveSubmenu в Sidebar.tsx. Обновить isArchiveActive для pathname /archive/timelines.</t>
+        </is>
+      </c>
+      <c r="E153" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F153" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G153" s="19" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="H153" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+      <c r="I153" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="20" customHeight="1" s="15">
+      <c r="A154" s="18" t="inlineStr">
+        <is>
+          <t>T-149</t>
+        </is>
+      </c>
+      <c r="B154" s="18" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C154" s="19" t="inlineStr">
+        <is>
+          <t>Frontend: навигация к видеозаписи при клике на красную колбаску</t>
+        </is>
+      </c>
+      <c r="D154" s="19" t="inlineStr">
+        <is>
+          <t>При клике на красную колбаску (has_recording=true) навигация на /archive/devices/:deviceId?session=:sessionId&amp;date=:date. Серые колбаски (has_recording=false) не кликабельны для видео.</t>
+        </is>
+      </c>
+      <c r="E154" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F154" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G154" s="19" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="H154" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+      <c r="I154" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="20" customHeight="1" s="15">
+      <c r="A155" s="18" t="inlineStr">
+        <is>
+          <t>T-150</t>
+        </is>
+      </c>
+      <c r="B155" s="18" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C155" s="19" t="inlineStr">
+        <is>
+          <t>Frontend: sidebar spacing -- отступ между пунктом и подменю</t>
+        </is>
+      </c>
+      <c r="D155" s="19" t="inlineStr">
+        <is>
+          <t>Добавить mt-1 div-обёртку к блокам подменю Аналитика и Настройки в Sidebar.tsx. 4 места: 2x SuperAdmin layout (строки 188, 212), 2x OAuth layout (строки 323, 347). Спецификация: docs/timelines-spec.md раздел 7</t>
+        </is>
+      </c>
+      <c r="E155" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F155" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G155" s="19" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="H155" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+      <c r="I155" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="20" customHeight="1" s="15">
+      <c r="A156" s="18" t="inlineStr">
+        <is>
+          <t>T-151</t>
+        </is>
+      </c>
+      <c r="B156" s="18" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C156" s="19" t="inlineStr">
+        <is>
+          <t>Frontend: заменить favicon на Кадеро</t>
+        </is>
+      </c>
+      <c r="D156" s="19" t="inlineStr">
+        <is>
+          <t>1. Скопировать assets/favicon.png в web-dashboard/public/favicon.png. 2. В index.html заменить link rel=icon с vite.svg на favicon.png (type=image/png). 3. Удалить web-dashboard/public/vite.svg. Спецификация: docs/timelines-spec.md раздел 8</t>
+        </is>
+      </c>
+      <c r="E156" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F156" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G156" s="19" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="H156" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+      <c r="I156" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="20" customHeight="1" s="15">
+      <c r="A157" s="18" t="inlineStr">
+        <is>
+          <t>T-152</t>
+        </is>
+      </c>
+      <c r="B157" s="18" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C157" s="19" t="inlineStr">
+        <is>
+          <t>Frontend: удалить Mail.ru OAuth из LoginPage, OAuthLoginPage, auth.ts</t>
+        </is>
+      </c>
+      <c r="D157" s="19" t="inlineStr">
+        <is>
+          <t>Удалить из auth.ts: функцию getMailruOAuthLoginUrl(). Из LoginPage.tsx: импорт getMailruOAuthLoginUrl, handleMailruLogin, кнопку 'Войти через Mail.ru'. Из OAuthLoginPage.tsx: импорт getMailruOAuthLoginUrl, handleMailruLogin, кнопку 'Войти через Mail.ru'. Спецификация: docs/timelines-spec.md раздел 9</t>
+        </is>
+      </c>
+      <c r="E157" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F157" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G157" s="19" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="H157" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+      <c r="I157" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="20" customHeight="1" s="15">
+      <c r="A158" s="18" t="inlineStr">
+        <is>
+          <t>T-153</t>
+        </is>
+      </c>
+      <c r="B158" s="18" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C158" s="19" t="inlineStr">
+        <is>
+          <t>Тестирование: endpoint /users/timeline с реальными данными</t>
+        </is>
+      </c>
+      <c r="D158" s="19" t="inlineStr">
+        <is>
+          <t>Функциональный тест на test-стейджинге: вызов GET /api/v1/ingest/users/timeline с JWT, проверка формата ответа, наличия пользователей, иерархии групп, has_recording флагов.</t>
+        </is>
+      </c>
+      <c r="E158" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F158" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G158" s="19" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="H158" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+      <c r="I158" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="20" customHeight="1" s="15">
+      <c r="A159" s="18" t="inlineStr">
+        <is>
+          <t>T-154</t>
+        </is>
+      </c>
+      <c r="B159" s="18" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C159" s="19" t="inlineStr">
+        <is>
+          <t>Тестирование: Yandex OAuth после удаления Mail.ru</t>
+        </is>
+      </c>
+      <c r="D159" s="19" t="inlineStr">
+        <is>
+          <t>Убедиться что Yandex OAuth продолжает работать: авторизация, callback, onboarding, select-tenant. Проверить что endpoints /mailru и /mailru/callback возвращают 404.</t>
+        </is>
+      </c>
+      <c r="E159" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F159" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G159" s="19" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="H159" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+      <c r="I159" s="18" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="20" customHeight="1" s="15">
+      <c r="A160" s="24" t="inlineStr">
+        <is>
+          <t>T-155</t>
+        </is>
+      </c>
+      <c r="B160" s="24" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C160" s="25" t="inlineStr">
+        <is>
+          <t>Crash на странице справочников: Cannot read properties of undefined (reading length)</t>
+        </is>
+      </c>
+      <c r="D160" s="25" t="inlineStr">
+        <is>
+          <t>Фронтенд ожидал объект-обёртку {groups: [], total: N} от API getGroups/getGroupItems, а backend возвращает List&lt;T&gt; (массив). resp.groups и resp.items возвращали undefined, вызывая TypeError при обращении к .length</t>
+        </is>
+      </c>
+      <c r="E160" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F160" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G160" s="25" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="H160" s="24" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+      <c r="I160" s="24" t="inlineStr">
         <is>
           <t>09.03.2026</t>
         </is>
@@ -7304,7 +8009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J97"/>
+  <dimension ref="A1:J113"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="15" min="1" max="1"/>
@@ -12167,6 +12872,838 @@
         </is>
       </c>
       <c r="J97" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="50" customHeight="1" s="15">
+      <c r="A98" s="22" t="inlineStr">
+        <is>
+          <t>TC-093</t>
+        </is>
+      </c>
+      <c r="B98" s="22" t="inlineStr">
+        <is>
+          <t>Agent Lifecycle</t>
+        </is>
+      </c>
+      <c r="C98" s="23" t="inlineStr">
+        <is>
+          <t>Heartbeat: все 9 валидных статусов принимаются (200)</t>
+        </is>
+      </c>
+      <c r="D98" s="23" t="inlineStr">
+        <is>
+          <t>Устройство 60b50ed1 зарегистрировано в тенанте Test Organization, JWT token user test</t>
+        </is>
+      </c>
+      <c r="E98" s="22" t="inlineStr">
+        <is>
+          <t>1. PUT /api/cp/v1/devices/{id}/heartbeat с status=starting\n2. Повторить для configuring, awaiting_user, idle, stopped, recording, online, error, offline\n3. Проверить HTTP 200 и корректный JSON response для каждого</t>
+        </is>
+      </c>
+      <c r="F98" s="22" t="inlineStr">
+        <is>
+          <t>Все 9 статусов возвращают HTTP 200, ответ содержит server_ts, pending_commands, next_heartbeat_sec, device_settings</t>
+        </is>
+      </c>
+      <c r="G98" s="23" t="inlineStr">
+        <is>
+          <t>Все 9 статусов (starting, configuring, awaiting_user, idle, stopped, recording, online, error, offline) возвращают HTTP 200 с корректным JSON</t>
+        </is>
+      </c>
+      <c r="H98" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I98" s="22" t="inlineStr">
+        <is>
+          <t>T-141</t>
+        </is>
+      </c>
+      <c r="J98" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="50" customHeight="1" s="15">
+      <c r="A99" s="22" t="inlineStr">
+        <is>
+          <t>TC-094</t>
+        </is>
+      </c>
+      <c r="B99" s="22" t="inlineStr">
+        <is>
+          <t>Agent Lifecycle</t>
+        </is>
+      </c>
+      <c r="C99" s="23" t="inlineStr">
+        <is>
+          <t>Heartbeat: структура ответа (server_ts, commands, settings, types)</t>
+        </is>
+      </c>
+      <c r="D99" s="23" t="inlineStr">
+        <is>
+          <t>Устройство 60b50ed1 зарегистрировано</t>
+        </is>
+      </c>
+      <c r="E99" s="22" t="inlineStr">
+        <is>
+          <t>1. PUT heartbeat со status=online\n2. Проверить наличие полей: server_ts (string ISO8601), pending_commands (array), next_heartbeat_sec (int), device_settings (object)\n3. Проверить device_settings содержит: fps (int), auto_start (bool), resolution (string), session_max_duration_hours (int)</t>
+        </is>
+      </c>
+      <c r="F99" s="22" t="inlineStr">
+        <is>
+          <t>Все поля присутствуют, типы корректны, server_ts в ISO 8601</t>
+        </is>
+      </c>
+      <c r="G99" s="23" t="inlineStr">
+        <is>
+          <t>server_ts (string ISO8601), pending_commands (array), next_heartbeat_sec=30 (int), device_settings: fps=1 (int), auto_start=true (bool), resolution=720p (string), session_max_duration_hours=24 (int)</t>
+        </is>
+      </c>
+      <c r="H99" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I99" s="22" t="inlineStr">
+        <is>
+          <t>T-141</t>
+        </is>
+      </c>
+      <c r="J99" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="50" customHeight="1" s="15">
+      <c r="A100" s="22" t="inlineStr">
+        <is>
+          <t>TC-095</t>
+        </is>
+      </c>
+      <c r="B100" s="22" t="inlineStr">
+        <is>
+          <t>Agent Lifecycle</t>
+        </is>
+      </c>
+      <c r="C100" s="23" t="inlineStr">
+        <is>
+          <t>Heartbeat: невалидный статус -&gt; 400 VALIDATION_ERROR</t>
+        </is>
+      </c>
+      <c r="D100" s="23" t="inlineStr">
+        <is>
+          <t>Устройство 60b50ed1 зарегистрировано</t>
+        </is>
+      </c>
+      <c r="E100" s="22" t="inlineStr">
+        <is>
+          <t>1. PUT heartbeat с status=INVALID_STATUS\n2. Проверить HTTP 400\n3. Проверить body содержит error и code=VALIDATION_ERROR</t>
+        </is>
+      </c>
+      <c r="F100" s="22" t="inlineStr">
+        <is>
+          <t>HTTP 400, body: {error: 'Invalid status value', code: 'VALIDATION_ERROR'}</t>
+        </is>
+      </c>
+      <c r="G100" s="23" t="inlineStr">
+        <is>
+          <t>HTTP 400, body: {error: 'Invalid status value', code: 'VALIDATION_ERROR'}</t>
+        </is>
+      </c>
+      <c r="H100" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I100" s="22" t="inlineStr">
+        <is>
+          <t>T-141</t>
+        </is>
+      </c>
+      <c r="J100" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="50" customHeight="1" s="15">
+      <c r="A101" s="22" t="inlineStr">
+        <is>
+          <t>TC-096</t>
+        </is>
+      </c>
+      <c r="B101" s="22" t="inlineStr">
+        <is>
+          <t>Agent Lifecycle</t>
+        </is>
+      </c>
+      <c r="C101" s="23" t="inlineStr">
+        <is>
+          <t>Heartbeat: пустое тело запроса -&gt; 400</t>
+        </is>
+      </c>
+      <c r="D101" s="23" t="inlineStr">
+        <is>
+          <t>Устройство 60b50ed1 зарегистрировано</t>
+        </is>
+      </c>
+      <c r="E101" s="22" t="inlineStr">
+        <is>
+          <t>1. PUT heartbeat с body {}\n2. Проверить HTTP 400</t>
+        </is>
+      </c>
+      <c r="F101" s="22" t="inlineStr">
+        <is>
+          <t>HTTP 400, body: {error: 'Status is required', code: 'VALIDATION_ERROR'}</t>
+        </is>
+      </c>
+      <c r="G101" s="23" t="inlineStr">
+        <is>
+          <t>HTTP 400, body: {error: 'Status is required', code: 'VALIDATION_ERROR'}</t>
+        </is>
+      </c>
+      <c r="H101" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I101" s="22" t="inlineStr">
+        <is>
+          <t>T-141</t>
+        </is>
+      </c>
+      <c r="J101" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="50" customHeight="1" s="15">
+      <c r="A102" s="22" t="inlineStr">
+        <is>
+          <t>TC-097</t>
+        </is>
+      </c>
+      <c r="B102" s="22" t="inlineStr">
+        <is>
+          <t>Agent Lifecycle</t>
+        </is>
+      </c>
+      <c r="C102" s="23" t="inlineStr">
+        <is>
+          <t>Heartbeat: без авторизации -&gt; 401 UNAUTHORIZED</t>
+        </is>
+      </c>
+      <c r="D102" s="23" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="E102" s="22" t="inlineStr">
+        <is>
+          <t>1. PUT heartbeat без заголовка Authorization\n2. Проверить HTTP 401</t>
+        </is>
+      </c>
+      <c r="F102" s="22" t="inlineStr">
+        <is>
+          <t>HTTP 401, body: {error: '...', code: 'UNAUTHORIZED'}</t>
+        </is>
+      </c>
+      <c r="G102" s="23" t="inlineStr">
+        <is>
+          <t>HTTP 401, body: {error: 'Missing or invalid Authorization header', code: 'UNAUTHORIZED'}</t>
+        </is>
+      </c>
+      <c r="H102" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I102" s="22" t="inlineStr">
+        <is>
+          <t>T-141</t>
+        </is>
+      </c>
+      <c r="J102" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="50" customHeight="1" s="15">
+      <c r="A103" s="22" t="inlineStr">
+        <is>
+          <t>TC-098</t>
+        </is>
+      </c>
+      <c r="B103" s="22" t="inlineStr">
+        <is>
+          <t>Agent Lifecycle</t>
+        </is>
+      </c>
+      <c r="C103" s="23" t="inlineStr">
+        <is>
+          <t>Heartbeat: cross-tenant device -&gt; 404 DEVICE_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="D103" s="23" t="inlineStr">
+        <is>
+          <t>Устройство 64b4d56e в тенанте Тест 1, JWT от user test (Test Organization)</t>
+        </is>
+      </c>
+      <c r="E103" s="22" t="inlineStr">
+        <is>
+          <t>1. PUT heartbeat для device 64b4d56e с токеном user test\n2. Проверить HTTP 404</t>
+        </is>
+      </c>
+      <c r="F103" s="22" t="inlineStr">
+        <is>
+          <t>HTTP 404, body: {error: 'Device not found: ...', code: 'DEVICE_NOT_FOUND'}</t>
+        </is>
+      </c>
+      <c r="G103" s="23" t="inlineStr">
+        <is>
+          <t>HTTP 404, body: {error: 'Device not found: 64b4d56e-...', code: 'DEVICE_NOT_FOUND'}</t>
+        </is>
+      </c>
+      <c r="H103" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I103" s="22" t="inlineStr">
+        <is>
+          <t>T-141</t>
+        </is>
+      </c>
+      <c r="J103" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="50" customHeight="1" s="15">
+      <c r="A104" s="22" t="inlineStr">
+        <is>
+          <t>TC-099</t>
+        </is>
+      </c>
+      <c r="B104" s="22" t="inlineStr">
+        <is>
+          <t>Agent Lifecycle</t>
+        </is>
+      </c>
+      <c r="C104" s="23" t="inlineStr">
+        <is>
+          <t>Heartbeat: session_locked=true принимается корректно</t>
+        </is>
+      </c>
+      <c r="D104" s="23" t="inlineStr">
+        <is>
+          <t>Устройство 60b50ed1 зарегистрировано</t>
+        </is>
+      </c>
+      <c r="E104" s="22" t="inlineStr">
+        <is>
+          <t>1. PUT heartbeat с session_locked=true, status=idle\n2. Проверить HTTP 200\n3. Проверить status-log: details содержит session_locked=true</t>
+        </is>
+      </c>
+      <c r="F104" s="22" t="inlineStr">
+        <is>
+          <t>HTTP 200, status-log entry details.session_locked=true</t>
+        </is>
+      </c>
+      <c r="G104" s="23" t="inlineStr">
+        <is>
+          <t>HTTP 200, status-log entry: details.session_locked=true, details.agent_version=1.0.0-test</t>
+        </is>
+      </c>
+      <c r="H104" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I104" s="22" t="inlineStr">
+        <is>
+          <t>T-141</t>
+        </is>
+      </c>
+      <c r="J104" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="50" customHeight="1" s="15">
+      <c r="A105" s="22" t="inlineStr">
+        <is>
+          <t>TC-100</t>
+        </is>
+      </c>
+      <c r="B105" s="22" t="inlineStr">
+        <is>
+          <t>Agent Lifecycle</t>
+        </is>
+      </c>
+      <c r="C105" s="23" t="inlineStr">
+        <is>
+          <t>Heartbeat: повторный heartbeat с тем же статусом не создает запись в status-log</t>
+        </is>
+      </c>
+      <c r="D105" s="23" t="inlineStr">
+        <is>
+          <t>Устройство 60b50ed1, текущий статус online</t>
+        </is>
+      </c>
+      <c r="E105" s="22" t="inlineStr">
+        <is>
+          <t>1. Запомнить total_elements в status-log\n2. PUT heartbeat с тем же status=online\n3. Проверить total_elements не изменился</t>
+        </is>
+      </c>
+      <c r="F105" s="22" t="inlineStr">
+        <is>
+          <t>total_elements до и после одинаков, дубликат не создан</t>
+        </is>
+      </c>
+      <c r="G105" s="23" t="inlineStr">
+        <is>
+          <t>total_elements=11 до и после повторного heartbeat с status=online, дубликат не создан</t>
+        </is>
+      </c>
+      <c r="H105" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I105" s="22" t="inlineStr">
+        <is>
+          <t>T-141</t>
+        </is>
+      </c>
+      <c r="J105" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="50" customHeight="1" s="15">
+      <c r="A106" s="22" t="inlineStr">
+        <is>
+          <t>TC-101</t>
+        </is>
+      </c>
+      <c r="B106" s="22" t="inlineStr">
+        <is>
+          <t>Agent Lifecycle</t>
+        </is>
+      </c>
+      <c r="C106" s="23" t="inlineStr">
+        <is>
+          <t>Status-Log: happy path - список переходов статусов</t>
+        </is>
+      </c>
+      <c r="D106" s="23" t="inlineStr">
+        <is>
+          <t>Устройство 60b50ed1, ранее выполнены heartbeat с разными статусами</t>
+        </is>
+      </c>
+      <c r="E106" s="22" t="inlineStr">
+        <is>
+          <t>1. GET /api/cp/v1/devices/{id}/status-log?page=0&amp;size=20\n2. Проверить HTTP 200\n3. Проверить структуру: content[], page, size, total_elements, total_pages\n4. Каждый элемент содержит: id, device_id, previous_status, new_status, changed_ts, trigger, details</t>
+        </is>
+      </c>
+      <c r="F106" s="22" t="inlineStr">
+        <is>
+          <t>HTTP 200, paginated response с корректной структурой, записи отсортированы по changed_ts DESC</t>
+        </is>
+      </c>
+      <c r="G106" s="23" t="inlineStr">
+        <is>
+          <t>HTTP 200, paginated: {content: [...], page: 0, size: 20, total_elements: 9, total_pages: 1}. Каждый элемент: id, device_id, previous_status, new_status, changed_ts, trigger=heartbeat, details</t>
+        </is>
+      </c>
+      <c r="H106" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I106" s="22" t="inlineStr">
+        <is>
+          <t>T-141</t>
+        </is>
+      </c>
+      <c r="J106" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="50" customHeight="1" s="15">
+      <c r="A107" s="22" t="inlineStr">
+        <is>
+          <t>TC-102</t>
+        </is>
+      </c>
+      <c r="B107" s="22" t="inlineStr">
+        <is>
+          <t>Agent Lifecycle</t>
+        </is>
+      </c>
+      <c r="C107" s="23" t="inlineStr">
+        <is>
+          <t>Status-Log: пагинация (page/size/total_pages)</t>
+        </is>
+      </c>
+      <c r="D107" s="23" t="inlineStr">
+        <is>
+          <t>Устройство 60b50ed1, минимум 9 записей в status-log</t>
+        </is>
+      </c>
+      <c r="E107" s="22" t="inlineStr">
+        <is>
+          <t>1. GET status-log?page=0&amp;size=3 -&gt; 3 записи, total_pages=N\n2. GET status-log?page=1&amp;size=3 -&gt; следующие 3 записи\n3. GET status-log?page=last&amp;size=3 -&gt; остаток записей\n4. Проверить что записи не дублируются между страницами</t>
+        </is>
+      </c>
+      <c r="F107" s="22" t="inlineStr">
+        <is>
+          <t>Пагинация корректна: total_elements совпадает, записи не дублируются, last page содержит остаток</t>
+        </is>
+      </c>
+      <c r="G107" s="23" t="inlineStr">
+        <is>
+          <t>page=0,size=3: 3 записи, total_pages=4. page=1,size=3: следующие 3. page=3,size=3: 2 остаточных записи. Записи не дублируются между страницами</t>
+        </is>
+      </c>
+      <c r="H107" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I107" s="22" t="inlineStr">
+        <is>
+          <t>T-141</t>
+        </is>
+      </c>
+      <c r="J107" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="50" customHeight="1" s="15">
+      <c r="A108" s="22" t="inlineStr">
+        <is>
+          <t>TC-103</t>
+        </is>
+      </c>
+      <c r="B108" s="22" t="inlineStr">
+        <is>
+          <t>Agent Lifecycle</t>
+        </is>
+      </c>
+      <c r="C108" s="23" t="inlineStr">
+        <is>
+          <t>Status-Log: фильтрация по дате (from/to)</t>
+        </is>
+      </c>
+      <c r="D108" s="23" t="inlineStr">
+        <is>
+          <t>Устройство 60b50ed1, записи с known timestamps</t>
+        </is>
+      </c>
+      <c r="E108" s="22" t="inlineStr">
+        <is>
+          <t>1. GET status-log?from=T1&amp;to=T2 где T1-T2 покрывает часть записей\n2. Проверить что возвращены только записи в диапазоне\n3. GET status-log?from=future_date -&gt; пустой результат\n4. Проверить HTTP 200 и total_elements=0</t>
+        </is>
+      </c>
+      <c r="F108" s="22" t="inlineStr">
+        <is>
+          <t>Фильтрация по дате корректна, пустой диапазон возвращает 0 записей с HTTP 200</t>
+        </is>
+      </c>
+      <c r="G108" s="23" t="inlineStr">
+        <is>
+          <t>from=...55Z&amp;to=...58Z: 4 записи в диапазоне. from=2027-01-01: 0 записей, HTTP 200, total_elements=0</t>
+        </is>
+      </c>
+      <c r="H108" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I108" s="22" t="inlineStr">
+        <is>
+          <t>T-141</t>
+        </is>
+      </c>
+      <c r="J108" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="50" customHeight="1" s="15">
+      <c r="A109" s="22" t="inlineStr">
+        <is>
+          <t>TC-104</t>
+        </is>
+      </c>
+      <c r="B109" s="22" t="inlineStr">
+        <is>
+          <t>Agent Lifecycle</t>
+        </is>
+      </c>
+      <c r="C109" s="23" t="inlineStr">
+        <is>
+          <t>Status-Log: несуществующее устройство -&gt; 404</t>
+        </is>
+      </c>
+      <c r="D109" s="23" t="inlineStr">
+        <is>
+          <t>Нет устройства с ID 00000000-0000-0000-0000-000000000000</t>
+        </is>
+      </c>
+      <c r="E109" s="22" t="inlineStr">
+        <is>
+          <t>1. GET status-log для device 00000000-0000-0000-0000-000000000000\n2. Проверить HTTP 404</t>
+        </is>
+      </c>
+      <c r="F109" s="22" t="inlineStr">
+        <is>
+          <t>HTTP 404, body: {error: 'Device not found: ...', code: 'DEVICE_NOT_FOUND'}</t>
+        </is>
+      </c>
+      <c r="G109" s="23" t="inlineStr">
+        <is>
+          <t>HTTP 404, body: {error: 'Device not found: 00000000-0000-0000-0000-000000000000', code: 'DEVICE_NOT_FOUND'}</t>
+        </is>
+      </c>
+      <c r="H109" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I109" s="22" t="inlineStr">
+        <is>
+          <t>T-141</t>
+        </is>
+      </c>
+      <c r="J109" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="50" customHeight="1" s="15">
+      <c r="A110" s="22" t="inlineStr">
+        <is>
+          <t>TC-105</t>
+        </is>
+      </c>
+      <c r="B110" s="22" t="inlineStr">
+        <is>
+          <t>Agent Lifecycle</t>
+        </is>
+      </c>
+      <c r="C110" s="23" t="inlineStr">
+        <is>
+          <t>Status-Log: без авторизации -&gt; 401</t>
+        </is>
+      </c>
+      <c r="D110" s="23" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="E110" s="22" t="inlineStr">
+        <is>
+          <t>1. GET status-log без заголовка Authorization\n2. Проверить HTTP 401</t>
+        </is>
+      </c>
+      <c r="F110" s="22" t="inlineStr">
+        <is>
+          <t>HTTP 401, body: {error: '...', code: 'UNAUTHORIZED'}</t>
+        </is>
+      </c>
+      <c r="G110" s="23" t="inlineStr">
+        <is>
+          <t>HTTP 401, body: {error: 'Missing or invalid Authorization header', code: 'UNAUTHORIZED'}</t>
+        </is>
+      </c>
+      <c r="H110" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I110" s="22" t="inlineStr">
+        <is>
+          <t>T-141</t>
+        </is>
+      </c>
+      <c r="J110" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="50" customHeight="1" s="15">
+      <c r="A111" s="22" t="inlineStr">
+        <is>
+          <t>TC-106</t>
+        </is>
+      </c>
+      <c r="B111" s="22" t="inlineStr">
+        <is>
+          <t>Agent Lifecycle</t>
+        </is>
+      </c>
+      <c r="C111" s="23" t="inlineStr">
+        <is>
+          <t>Status-Log: cross-tenant device -&gt; 404 (tenant isolation)</t>
+        </is>
+      </c>
+      <c r="D111" s="23" t="inlineStr">
+        <is>
+          <t>Устройство 64b4d56e в тенанте Тест 1, JWT user test из Test Organization</t>
+        </is>
+      </c>
+      <c r="E111" s="22" t="inlineStr">
+        <is>
+          <t>1. GET status-log для device 64b4d56e с токеном user test\n2. Проверить HTTP 404 (не 403)</t>
+        </is>
+      </c>
+      <c r="F111" s="22" t="inlineStr">
+        <is>
+          <t>HTTP 404, code: DEVICE_NOT_FOUND. Тенантная изоляция: устройство не видно из другого тенанта</t>
+        </is>
+      </c>
+      <c r="G111" s="23" t="inlineStr">
+        <is>
+          <t>HTTP 404, body: {error: 'Device not found: 64b4d56e-...', code: 'DEVICE_NOT_FOUND'}. Тенантная изоляция работает: 404, а не 403</t>
+        </is>
+      </c>
+      <c r="H111" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I111" s="22" t="inlineStr">
+        <is>
+          <t>T-141</t>
+        </is>
+      </c>
+      <c r="J111" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="50" customHeight="1" s="15">
+      <c r="A112" s="22" t="inlineStr">
+        <is>
+          <t>TC-107</t>
+        </is>
+      </c>
+      <c r="B112" s="22" t="inlineStr">
+        <is>
+          <t>Agent Lifecycle</t>
+        </is>
+      </c>
+      <c r="C112" s="23" t="inlineStr">
+        <is>
+          <t>Device Settings: heartbeat возвращает корректные настройки устройства</t>
+        </is>
+      </c>
+      <c r="D112" s="23" t="inlineStr">
+        <is>
+          <t>Устройство 60b50ed1 с сохраненными settings</t>
+        </is>
+      </c>
+      <c r="E112" s="22" t="inlineStr">
+        <is>
+          <t>1. GET device details -&gt; запомнить settings\n2. PUT heartbeat\n3. Сравнить device_settings из heartbeat response с settings из device details\n4. Проверить fps=1, resolution=720p</t>
+        </is>
+      </c>
+      <c r="F112" s="22" t="inlineStr">
+        <is>
+          <t>device_settings в heartbeat совпадают с settings устройства в БД, fps=1, resolution=720p</t>
+        </is>
+      </c>
+      <c r="G112" s="23" t="inlineStr">
+        <is>
+          <t>device_settings из heartbeat: {fps:1, auto_start:true, resolution:720p, session_max_duration_hours:24} совпадает с settings устройства из GET /devices/{id}</t>
+        </is>
+      </c>
+      <c r="H112" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I112" s="22" t="inlineStr">
+        <is>
+          <t>T-141</t>
+        </is>
+      </c>
+      <c r="J112" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="50" customHeight="1" s="15">
+      <c r="A113" s="22" t="inlineStr">
+        <is>
+          <t>TC-108</t>
+        </is>
+      </c>
+      <c r="B113" s="22" t="inlineStr">
+        <is>
+          <t>Agent Lifecycle</t>
+        </is>
+      </c>
+      <c r="C113" s="23" t="inlineStr">
+        <is>
+          <t>Auth-service: дефолты device settings (capture_fps=1, auto_start=false, resolution=720p)</t>
+        </is>
+      </c>
+      <c r="D113" s="23" t="inlineStr">
+        <is>
+          <t>Код auth-service проверен, application.yml без overrides</t>
+        </is>
+      </c>
+      <c r="E113" s="22" t="inlineStr">
+        <is>
+          <t>1. Проверить @Value аннотации в DeviceAuthService\n2. Дефолты: capture-fps=1, quality=low, default-resolution=720p, segment-duration-sec=60, default-session-max-min=60, default-session-max-hours=0, default-auto-start=false</t>
+        </is>
+      </c>
+      <c r="F113" s="22" t="inlineStr">
+        <is>
+          <t>Дефолты соответствуют спецификации: fps=1, quality=low, resolution=720p, segment_duration=60s, session_max=60min, auto_start=false</t>
+        </is>
+      </c>
+      <c r="G113" s="23" t="inlineStr">
+        <is>
+          <t>Код DeviceAuthService проверен. @Value дефолты: capture-fps=1, quality=low, default-resolution=720p, segment-duration-sec=60, default-session-max-min=60, default-session-max-hours=0, default-auto-start=false. Соответствует спецификации</t>
+        </is>
+      </c>
+      <c r="H113" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I113" s="22" t="inlineStr">
+        <is>
+          <t>T-141</t>
+        </is>
+      </c>
+      <c r="J113" s="23" t="inlineStr">
         <is>
           <t>09.03.2026</t>
         </is>

</xml_diff>

<commit_message>
chore: add T-161..T-163 bugs and TC-130..TC-132 test cases
Dashboard SQL date bug, timeline recording correlation,
and invisible app group bars — all fixed and verified on test.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracker.xlsx
+++ b/docs/tracker.xlsx
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I160"/>
+  <dimension ref="A1:I168"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="15" min="1" max="1"/>
@@ -7995,6 +7995,382 @@
         </is>
       </c>
     </row>
+    <row r="161" ht="20" customHeight="1" s="15">
+      <c r="A161" s="24" t="inlineStr">
+        <is>
+          <t>T-156</t>
+        </is>
+      </c>
+      <c r="B161" s="24" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C161" s="25" t="inlineStr">
+        <is>
+          <t>Timeline: невалидная дата возвращает 500 вместо 400</t>
+        </is>
+      </c>
+      <c r="D161" s="25" t="inlineStr">
+        <is>
+          <t>GET /api/v1/ingest/users/timeline?date=invalid возвращает 500 Internal Server Error вместо 400 Bad Request. Сервер не валидирует формат даты в query param date и необработанное исключение парсинга пробрасывается как 500. Необходимо добавить try-catch при парсинге LocalDate и возвращать 400 с информативным сообщением. Среда: test. Связанный тест: TC-111.</t>
+        </is>
+      </c>
+      <c r="E161" s="24" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F161" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G161" s="25" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="H161" s="24" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+      <c r="I161" s="24" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="20" customHeight="1" s="15">
+      <c r="A162" s="24" t="inlineStr">
+        <is>
+          <t>T-157</t>
+        </is>
+      </c>
+      <c r="B162" s="24" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C162" s="25" t="inlineStr">
+        <is>
+          <t>Catalogs: SUPER_ADMIN без tenant_id получает 500 (null tenant)</t>
+        </is>
+      </c>
+      <c r="D162" s="25" t="inlineStr">
+        <is>
+          <t>GET /api/v1/ingest/catalogs/groups?group_type=APP от SUPER_ADMIN (scope=global) без явного tenant_id возвращает 500. Причина: resolveEffectiveTenantId() при scope=global возвращает tenantIdParam as-is, который null. CatalogService.getGroups(null, ...) вызывает seed(null, ...) -&gt; INSERT с tenant_id=null -&gt; PSQLException: not-null constraint violation на app_groups.tenant_id. Workaround: передавать tenant_id явно. Fix: в resolveEffectiveTenantId при global scope если tenantIdParam=null, использовать principal.getTenantId() как fallback, либо возвращать 400 'tenant_id is required for global scope'. Среда: test. Связанные тесты: TC-114, TC-115.</t>
+        </is>
+      </c>
+      <c r="E162" s="24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F162" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G162" s="25" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="H162" s="24" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+      <c r="I162" s="24" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="20" customHeight="1" s="15">
+      <c r="A163" s="24" t="inlineStr">
+        <is>
+          <t>T-158</t>
+        </is>
+      </c>
+      <c r="B163" s="24" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C163" s="25" t="inlineStr">
+        <is>
+          <t>Timeline SQL: неверная нижняя граница date AT TIME ZONE отрезает 0-6ч MSK</t>
+        </is>
+      </c>
+      <c r="D163" s="25" t="inlineStr">
+        <is>
+          <t>В TimelineService.queryFocusIntervals SQL-выражение CAST(:date AS date) AT TIME ZONE :tz возвращает timestamp without time zone (не timestamptz), из-за чего PostgreSQL интерпретирует границу как UTC, а не как московское время. Для date=2026-03-09 tz=Europe/Moscow: фактическая нижняя граница = 06:00 MSK вместо 00:00 MSK. Данные с 00:00 до 06:00 MSK не попадают в выборку. Файл: TimelineService.java, строка 77.</t>
+        </is>
+      </c>
+      <c r="E163" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F163" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G163" s="25" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="H163" s="24" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+      <c r="I163" s="24" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="20" customHeight="1" s="15">
+      <c r="A164" s="24" t="inlineStr">
+        <is>
+          <t>T-159</t>
+        </is>
+      </c>
+      <c r="B164" s="24" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C164" s="25" t="inlineStr">
+        <is>
+          <t>Focus intervals: session_id всегда NULL — красные участки не отображаются</t>
+        </is>
+      </c>
+      <c r="D164" s="25" t="inlineStr">
+        <is>
+          <t>В таблице app_focus_intervals session_id = NULL для 100% записей (400 из 400). Агент передаёт sessionId = _commandHandler.CurrentSessionId, но это значение = null, если запись (recording) была запущена не командой START_RECORDING, а автоматически. При автозапуске записи SessionManager._currentSessionId заполняется, но ActiveWindowTracker/TrayWindowTracker может получать его с задержкой или из другого потока. Из-за отсутствия session_id backend не может определить has_recording=true, и красные полоски не отображаются. Файл: ActiveWindowTracker.cs:138, SessionManager.cs:49.</t>
+        </is>
+      </c>
+      <c r="E164" s="24" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F164" s="24" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G164" s="25" t="inlineStr">
+        <is>
+          <t>Алексей</t>
+        </is>
+      </c>
+      <c r="H164" s="24" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+      <c r="I164" s="24" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" ht="20" customHeight="1" s="15">
+      <c r="A165" s="24" t="inlineStr">
+        <is>
+          <t>T-160</t>
+        </is>
+      </c>
+      <c r="B165" s="24" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C165" s="25" t="inlineStr">
+        <is>
+          <t>Timeline: пользователи без focus intervals не отображаются (только из focusRows)</t>
+        </is>
+      </c>
+      <c r="D165" s="25" t="inlineStr">
+        <is>
+          <t>TimelineService.assembleTimeline() собирает пользователей ТОЛЬКО из focusRows (строка 179: byUser.entrySet()). Комментарий на строке 176 'Also include users from userInfoMap that might not have focus data' не реализован — код итерирует только byUser, игнорируя пользователей из device_user_sessions без focus данных. Если пользователь залогинен на устройстве, но не имеет focus intervals за выбранный день, он не попадёт в таймлайн.</t>
+        </is>
+      </c>
+      <c r="E165" s="24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F165" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G165" s="25" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="H165" s="24" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+      <c r="I165" s="24" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="20" customHeight="1" s="15">
+      <c r="A166" s="24" t="inlineStr">
+        <is>
+          <t>T-161</t>
+        </is>
+      </c>
+      <c r="B166" s="24" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C166" s="25" t="inlineStr">
+        <is>
+          <t>Dashboard графики не отображают данные (SQL date cast + DTO mismatch)</t>
+        </is>
+      </c>
+      <c r="D166" s="25" t="inlineStr">
+        <is>
+          <t>1. SQL: CAST(:from AS date) возвращает неверные границы дат → данные не попадают в выборку. Fix: CAST(:from AS timestamp). 2. DTO GroupInfo имел поля id/name, а фронт ожидал group_id/group_name (Jackson SNAKE_CASE). 3. Ungrouped данные (default group) не выделялись отдельно.</t>
+        </is>
+      </c>
+      <c r="E166" s="24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F166" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G166" s="25" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="H166" s="24" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+      <c r="I166" s="24" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" ht="20" customHeight="1" s="15">
+      <c r="A167" s="24" t="inlineStr">
+        <is>
+          <t>T-162</t>
+        </is>
+      </c>
+      <c r="B167" s="24" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C167" s="25" t="inlineStr">
+        <is>
+          <t>Timeline: нет информации о записях (server-side корреляция)</t>
+        </is>
+      </c>
+      <c r="D167" s="25" t="inlineStr">
+        <is>
+          <t>Timeline API не проверял наличие recording_sessions для каждого часа. Fix: добавлен запрос к recording_sessions + корреляция по device_id + overlap часа. has_recording и recording_session_ids теперь заполняются корректно.</t>
+        </is>
+      </c>
+      <c r="E167" s="24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F167" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G167" s="25" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="H167" s="24" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+      <c r="I167" s="24" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="20" customHeight="1" s="15">
+      <c r="A168" s="24" t="inlineStr">
+        <is>
+          <t>T-163</t>
+        </is>
+      </c>
+      <c r="B168" s="24" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C168" s="25" t="inlineStr">
+        <is>
+          <t>Timeline: невидимые bars групп приложений и нет bars для отдельных приложений</t>
+        </is>
+      </c>
+      <c r="D168" s="25" t="inlineStr">
+        <is>
+          <t>1. HourCells использовал colorClass=opacity-70 (нет фона → невидимые бары). Fix: inline style с backgroundColor. 2. Строки отдельных приложений имели пустые div без данных. Fix: добавлен расчёт per-hour per-app данных и рендеринг HourCells для всех уровней drill-down.</t>
+        </is>
+      </c>
+      <c r="E168" s="24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F168" s="24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G168" s="25" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="H168" s="24" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+      <c r="I168" s="24" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
@@ -8009,7 +8385,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J113"/>
+  <dimension ref="A1:J137"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="15" min="1" max="1"/>
@@ -13706,6 +14082,1250 @@
       <c r="J113" s="23" t="inlineStr">
         <is>
           <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="50" customHeight="1" s="15">
+      <c r="A114" s="22" t="inlineStr">
+        <is>
+          <t>TC-109</t>
+        </is>
+      </c>
+      <c r="B114" s="22" t="inlineStr">
+        <is>
+          <t>Timeline API</t>
+        </is>
+      </c>
+      <c r="C114" s="23" t="inlineStr">
+        <is>
+          <t>Timeline endpoint - happy path (сегодня)</t>
+        </is>
+      </c>
+      <c r="D114" s="23" t="inlineStr">
+        <is>
+          <t>JWT superadmin, test-стейджинг</t>
+        </is>
+      </c>
+      <c r="E114" s="22" t="inlineStr">
+        <is>
+          <t>1. GET /users/timeline?date=&lt;today&gt;\n2. Проверить HTTP 200\n3. Проверить JSON: date, timezone, users[]</t>
+        </is>
+      </c>
+      <c r="F114" s="22" t="inlineStr">
+        <is>
+          <t>200, JSON с полями date, timezone, users[]</t>
+        </is>
+      </c>
+      <c r="G114" s="23" t="inlineStr">
+        <is>
+          <t>200, JSON: date=2026-03-09, timezone=Europe/Moscow, users[] с 2 пользователями, hours[] с app_groups[]</t>
+        </is>
+      </c>
+      <c r="H114" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I114" s="22" t="inlineStr">
+        <is>
+          <t>T-142</t>
+        </is>
+      </c>
+      <c r="J114" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="50" customHeight="1" s="15">
+      <c r="A115" s="22" t="inlineStr">
+        <is>
+          <t>TC-110</t>
+        </is>
+      </c>
+      <c r="B115" s="22" t="inlineStr">
+        <is>
+          <t>Timeline API</t>
+        </is>
+      </c>
+      <c r="C115" s="23" t="inlineStr">
+        <is>
+          <t>Timeline endpoint - конкретная дата 2026-03-09</t>
+        </is>
+      </c>
+      <c r="D115" s="23" t="inlineStr">
+        <is>
+          <t>JWT superadmin, test-стейджинг</t>
+        </is>
+      </c>
+      <c r="E115" s="22" t="inlineStr">
+        <is>
+          <t>1. GET /users/timeline?date=2026-03-09\n2. Проверить HTTP 200\n3. Проверить JSON структуру</t>
+        </is>
+      </c>
+      <c r="F115" s="22" t="inlineStr">
+        <is>
+          <t>200, JSON</t>
+        </is>
+      </c>
+      <c r="G115" s="23" t="inlineStr">
+        <is>
+          <t>200, JSON: date=2026-03-09, timezone=Europe/Moscow, users[] с 2 пользователями и корректными данными</t>
+        </is>
+      </c>
+      <c r="H115" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I115" s="22" t="inlineStr">
+        <is>
+          <t>T-142</t>
+        </is>
+      </c>
+      <c r="J115" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="50" customHeight="1" s="15">
+      <c r="A116" s="22" t="inlineStr">
+        <is>
+          <t>TC-111</t>
+        </is>
+      </c>
+      <c r="B116" s="22" t="inlineStr">
+        <is>
+          <t>Timeline API</t>
+        </is>
+      </c>
+      <c r="C116" s="23" t="inlineStr">
+        <is>
+          <t>Timeline endpoint - невалидная дата</t>
+        </is>
+      </c>
+      <c r="D116" s="23" t="inlineStr">
+        <is>
+          <t>JWT superadmin, test-стейджинг</t>
+        </is>
+      </c>
+      <c r="E116" s="22" t="inlineStr">
+        <is>
+          <t>1. GET /users/timeline?date=invalid\n2. Проверить HTTP 400</t>
+        </is>
+      </c>
+      <c r="F116" s="22" t="inlineStr">
+        <is>
+          <t>400 Bad Request</t>
+        </is>
+      </c>
+      <c r="G116" s="23" t="inlineStr">
+        <is>
+          <t>400 Bad Request с сообщением 'Invalid date format: invalid. Expected: yyyy-MM-dd' (после фикса T-156)</t>
+        </is>
+      </c>
+      <c r="H116" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I116" s="22" t="inlineStr">
+        <is>
+          <t>T-142</t>
+        </is>
+      </c>
+      <c r="J116" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="50" customHeight="1" s="15">
+      <c r="A117" s="22" t="inlineStr">
+        <is>
+          <t>TC-112</t>
+        </is>
+      </c>
+      <c r="B117" s="22" t="inlineStr">
+        <is>
+          <t>Timeline API</t>
+        </is>
+      </c>
+      <c r="C117" s="23" t="inlineStr">
+        <is>
+          <t>Timeline endpoint - без авторизации</t>
+        </is>
+      </c>
+      <c r="D117" s="23" t="inlineStr">
+        <is>
+          <t>Без JWT, test-стейджинг</t>
+        </is>
+      </c>
+      <c r="E117" s="22" t="inlineStr">
+        <is>
+          <t>1. GET /users/timeline?date=2026-03-09 без Authorization header\n2. Проверить HTTP 401</t>
+        </is>
+      </c>
+      <c r="F117" s="22" t="inlineStr">
+        <is>
+          <t>401 Unauthorized</t>
+        </is>
+      </c>
+      <c r="G117" s="23" t="inlineStr">
+        <is>
+          <t>401 с {error:Missing or invalid Authorization header,code:MISSING_TOKEN}</t>
+        </is>
+      </c>
+      <c r="H117" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I117" s="22" t="inlineStr">
+        <is>
+          <t>T-142</t>
+        </is>
+      </c>
+      <c r="J117" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="50" customHeight="1" s="15">
+      <c r="A118" s="22" t="inlineStr">
+        <is>
+          <t>TC-113</t>
+        </is>
+      </c>
+      <c r="B118" s="22" t="inlineStr">
+        <is>
+          <t>Timeline API</t>
+        </is>
+      </c>
+      <c r="C118" s="23" t="inlineStr">
+        <is>
+          <t>Timeline endpoint - с таймзоной UTC</t>
+        </is>
+      </c>
+      <c r="D118" s="23" t="inlineStr">
+        <is>
+          <t>JWT superadmin, test-стейджинг</t>
+        </is>
+      </c>
+      <c r="E118" s="22" t="inlineStr">
+        <is>
+          <t>1. GET /users/timeline?date=2026-03-09&amp;timezone=UTC\n2. Проверить HTTP 200\n3. Проверить timezone в ответе</t>
+        </is>
+      </c>
+      <c r="F118" s="22" t="inlineStr">
+        <is>
+          <t>200, JSON с timezone=UTC</t>
+        </is>
+      </c>
+      <c r="G118" s="23" t="inlineStr">
+        <is>
+          <t>200, JSON: timezone=UTC, часы сдвинуты на -3 от Europe/Moscow (hour 10 MSK = hour 7 UTC). Конверсия таймзон работает корректно.</t>
+        </is>
+      </c>
+      <c r="H118" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I118" s="22" t="inlineStr">
+        <is>
+          <t>T-142</t>
+        </is>
+      </c>
+      <c r="J118" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="50" customHeight="1" s="15">
+      <c r="A119" s="22" t="inlineStr">
+        <is>
+          <t>TC-114</t>
+        </is>
+      </c>
+      <c r="B119" s="22" t="inlineStr">
+        <is>
+          <t>Catalogs API</t>
+        </is>
+      </c>
+      <c r="C119" s="23" t="inlineStr">
+        <is>
+          <t>Группы приложений - список (fix TypeError length)</t>
+        </is>
+      </c>
+      <c r="D119" s="23" t="inlineStr">
+        <is>
+          <t>JWT superadmin, test-стейджинг, T-155 исправлен</t>
+        </is>
+      </c>
+      <c r="E119" s="22" t="inlineStr">
+        <is>
+          <t>1. GET /catalogs/groups?type=APP\n2. Проверить HTTP 200\n3. Проверить что ответ - JSON массив</t>
+        </is>
+      </c>
+      <c r="F119" s="22" t="inlineStr">
+        <is>
+          <t>200, JSON массив (НЕ обертка)</t>
+        </is>
+      </c>
+      <c r="G119" s="23" t="inlineStr">
+        <is>
+          <t>400 Bad Request с 'tenant_id is required for global scope' при запросе без tenant_id. С tenant_id — 200, 9 групп (после фикса T-157)</t>
+        </is>
+      </c>
+      <c r="H119" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I119" s="22" t="inlineStr">
+        <is>
+          <t>T-155</t>
+        </is>
+      </c>
+      <c r="J119" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="50" customHeight="1" s="15">
+      <c r="A120" s="22" t="inlineStr">
+        <is>
+          <t>TC-115</t>
+        </is>
+      </c>
+      <c r="B120" s="22" t="inlineStr">
+        <is>
+          <t>Catalogs API</t>
+        </is>
+      </c>
+      <c r="C120" s="23" t="inlineStr">
+        <is>
+          <t>Группы сайтов - список</t>
+        </is>
+      </c>
+      <c r="D120" s="23" t="inlineStr">
+        <is>
+          <t>JWT superadmin, test-стейджинг</t>
+        </is>
+      </c>
+      <c r="E120" s="22" t="inlineStr">
+        <is>
+          <t>1. GET /catalogs/groups?type=SITE\n2. Проверить HTTP 200\n3. Проверить что ответ - JSON массив</t>
+        </is>
+      </c>
+      <c r="F120" s="22" t="inlineStr">
+        <is>
+          <t>200, JSON массив</t>
+        </is>
+      </c>
+      <c r="G120" s="23" t="inlineStr">
+        <is>
+          <t>400 Bad Request с 'tenant_id is required for global scope' при запросе без tenant_id. С tenant_id — 200, 13 групп (после фикса T-157)</t>
+        </is>
+      </c>
+      <c r="H120" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I120" s="22" t="inlineStr">
+        <is>
+          <t>T-155</t>
+        </is>
+      </c>
+      <c r="J120" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="50" customHeight="1" s="15">
+      <c r="A121" s="22" t="inlineStr">
+        <is>
+          <t>TC-116</t>
+        </is>
+      </c>
+      <c r="B121" s="22" t="inlineStr">
+        <is>
+          <t>OAuth</t>
+        </is>
+      </c>
+      <c r="C121" s="23" t="inlineStr">
+        <is>
+          <t>Mail.ru OAuth endpoint удален</t>
+        </is>
+      </c>
+      <c r="D121" s="23" t="inlineStr">
+        <is>
+          <t>test-стейджинг, Mail.ru OAuth удален из auth-service</t>
+        </is>
+      </c>
+      <c r="E121" s="22" t="inlineStr">
+        <is>
+          <t>1. GET /api/v1/auth/oauth/mailru\n2. Проверить что НЕ 200/302</t>
+        </is>
+      </c>
+      <c r="F121" s="22" t="inlineStr">
+        <is>
+          <t>404 или 401 (НЕ 200/302)</t>
+        </is>
+      </c>
+      <c r="G121" s="23" t="inlineStr">
+        <is>
+          <t>401 с {error:Authentication required,code:UNAUTHORIZED}. Endpoint недоступен - Mail.ru OAuth удален.</t>
+        </is>
+      </c>
+      <c r="H121" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I121" s="22" t="inlineStr">
+        <is>
+          <t>T-145</t>
+        </is>
+      </c>
+      <c r="J121" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="50" customHeight="1" s="15">
+      <c r="A122" s="22" t="inlineStr">
+        <is>
+          <t>TC-117</t>
+        </is>
+      </c>
+      <c r="B122" s="22" t="inlineStr">
+        <is>
+          <t>OAuth</t>
+        </is>
+      </c>
+      <c r="C122" s="23" t="inlineStr">
+        <is>
+          <t>Mail.ru callback удален</t>
+        </is>
+      </c>
+      <c r="D122" s="23" t="inlineStr">
+        <is>
+          <t>test-стейджинг, Mail.ru OAuth удален</t>
+        </is>
+      </c>
+      <c r="E122" s="22" t="inlineStr">
+        <is>
+          <t>1. GET /api/v1/auth/oauth/mailru/callback?code=test&amp;state=test\n2. Проверить что НЕ 200/302</t>
+        </is>
+      </c>
+      <c r="F122" s="22" t="inlineStr">
+        <is>
+          <t>404 или 401</t>
+        </is>
+      </c>
+      <c r="G122" s="23" t="inlineStr">
+        <is>
+          <t>401 с {error:Authentication required,code:UNAUTHORIZED}. Callback endpoint недоступен - Mail.ru OAuth удален.</t>
+        </is>
+      </c>
+      <c r="H122" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I122" s="22" t="inlineStr">
+        <is>
+          <t>T-145</t>
+        </is>
+      </c>
+      <c r="J122" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="50" customHeight="1" s="15">
+      <c r="A123" s="22" t="inlineStr">
+        <is>
+          <t>TC-118</t>
+        </is>
+      </c>
+      <c r="B123" s="22" t="inlineStr">
+        <is>
+          <t>OAuth</t>
+        </is>
+      </c>
+      <c r="C123" s="23" t="inlineStr">
+        <is>
+          <t>Yandex OAuth все еще работает</t>
+        </is>
+      </c>
+      <c r="D123" s="23" t="inlineStr">
+        <is>
+          <t>test-стейджинг</t>
+        </is>
+      </c>
+      <c r="E123" s="22" t="inlineStr">
+        <is>
+          <t>1. GET /api/v1/auth/oauth/yandex\n2. Проверить HTTP 200 или 302</t>
+        </is>
+      </c>
+      <c r="F123" s="22" t="inlineStr">
+        <is>
+          <t>200 или 302 (redirect к Яндексу)</t>
+        </is>
+      </c>
+      <c r="G123" s="23" t="inlineStr">
+        <is>
+          <t>302 redirect. Yandex OAuth работает, возвращает redirect к Яндексу.</t>
+        </is>
+      </c>
+      <c r="H123" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I123" s="22" t="inlineStr">
+        <is>
+          <t>T-145</t>
+        </is>
+      </c>
+      <c r="J123" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="50" customHeight="1" s="15">
+      <c r="A124" s="22" t="inlineStr">
+        <is>
+          <t>TC-119</t>
+        </is>
+      </c>
+      <c r="B124" s="22" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C124" s="23" t="inlineStr">
+        <is>
+          <t>Favicon загружается (favicon.png)</t>
+        </is>
+      </c>
+      <c r="D124" s="23" t="inlineStr">
+        <is>
+          <t>test-стейджинг</t>
+        </is>
+      </c>
+      <c r="E124" s="22" t="inlineStr">
+        <is>
+          <t>1. GET /screenrecorder/favicon.png\n2. Проверить HTTP 200</t>
+        </is>
+      </c>
+      <c r="F124" s="22" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G124" s="23" t="inlineStr">
+        <is>
+          <t>200. Favicon загружается корректно.</t>
+        </is>
+      </c>
+      <c r="H124" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I124" s="22" t="inlineStr">
+        <is>
+          <t>T-151</t>
+        </is>
+      </c>
+      <c r="J124" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="50" customHeight="1" s="15">
+      <c r="A125" s="22" t="inlineStr">
+        <is>
+          <t>TC-120</t>
+        </is>
+      </c>
+      <c r="B125" s="22" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C125" s="23" t="inlineStr">
+        <is>
+          <t>SPA загружается</t>
+        </is>
+      </c>
+      <c r="D125" s="23" t="inlineStr">
+        <is>
+          <t>test-стейджинг</t>
+        </is>
+      </c>
+      <c r="E125" s="22" t="inlineStr">
+        <is>
+          <t>1. GET /screenrecorder/\n2. Проверить HTTP 200</t>
+        </is>
+      </c>
+      <c r="F125" s="22" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G125" s="23" t="inlineStr">
+        <is>
+          <t>200. SPA загружается корректно.</t>
+        </is>
+      </c>
+      <c r="H125" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I125" s="22" t="inlineStr">
+        <is>
+          <t>T-151</t>
+        </is>
+      </c>
+      <c r="J125" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="50" customHeight="1" s="15">
+      <c r="A126" s="22" t="inlineStr">
+        <is>
+          <t>TC-121</t>
+        </is>
+      </c>
+      <c r="B126" s="22" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="C126" s="23" t="inlineStr">
+        <is>
+          <t>HTML содержит favicon.png (не vite.svg)</t>
+        </is>
+      </c>
+      <c r="D126" s="23" t="inlineStr">
+        <is>
+          <t>test-стейджинг</t>
+        </is>
+      </c>
+      <c r="E126" s="22" t="inlineStr">
+        <is>
+          <t>1. GET /screenrecorder/\n2. Найти в HTML favicon.png\n3. Убедиться что нет vite.svg</t>
+        </is>
+      </c>
+      <c r="F126" s="22" t="inlineStr">
+        <is>
+          <t>favicon.png найден, vite.svg отсутствует</t>
+        </is>
+      </c>
+      <c r="G126" s="23" t="inlineStr">
+        <is>
+          <t>favicon.png найден в HTML, vite.svg отсутствует.</t>
+        </is>
+      </c>
+      <c r="H126" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I126" s="22" t="inlineStr">
+        <is>
+          <t>T-151</t>
+        </is>
+      </c>
+      <c r="J126" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="50" customHeight="1" s="15">
+      <c r="A127" s="22" t="inlineStr">
+        <is>
+          <t>TC-122</t>
+        </is>
+      </c>
+      <c r="B127" s="22" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="C127" s="23" t="inlineStr">
+        <is>
+          <t>Login superadmin работает</t>
+        </is>
+      </c>
+      <c r="D127" s="23" t="inlineStr">
+        <is>
+          <t>test-стейджинг</t>
+        </is>
+      </c>
+      <c r="E127" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /api/v1/auth/login с superadmin/Admin@12345\n2. Проверить HTTP 200\n3. Проверить наличие access_token в ответе</t>
+        </is>
+      </c>
+      <c r="F127" s="22" t="inlineStr">
+        <is>
+          <t>200, JSON с access_token</t>
+        </is>
+      </c>
+      <c r="G127" s="23" t="inlineStr">
+        <is>
+          <t>200, JSON с access_token (1399 символов), user object с roles=[SUPER_ADMIN], 38 permissions.</t>
+        </is>
+      </c>
+      <c r="H127" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I127" s="22" t="inlineStr">
+        <is>
+          <t>T-153</t>
+        </is>
+      </c>
+      <c r="J127" s="23" t="inlineStr">
+        <is>
+          <t>09.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="50" customHeight="1" s="15">
+      <c r="A128" s="22" t="inlineStr">
+        <is>
+          <t>TC-123</t>
+        </is>
+      </c>
+      <c r="B128" s="22" t="inlineStr">
+        <is>
+          <t>Timeline</t>
+        </is>
+      </c>
+      <c r="C128" s="23" t="inlineStr">
+        <is>
+          <t>Timeline - правильные данные за все часы дня (T-158 fix)</t>
+        </is>
+      </c>
+      <c r="D128" s="23" t="inlineStr">
+        <is>
+          <t>Деплой с фиксом T-158 на test. Пользователь air911d\shepaland имеет данные за 2026-03-09</t>
+        </is>
+      </c>
+      <c r="E128" s="22" t="inlineStr">
+        <is>
+          <t>1. Авторизоваться superadmin\n2. GET /users/timeline?date=2026-03-09&amp;timezone=Europe/Moscow&amp;tenant_id=...\n3. Проверить что hours содержат данные за все часы с активностью\n4. Проверить has_recording и recording_session_ids</t>
+        </is>
+      </c>
+      <c r="F128" s="22" t="inlineStr">
+        <is>
+          <t>Пользователи с focus intervals отображаются, hours содержат корректные данные за все часы дня</t>
+        </is>
+      </c>
+      <c r="G128" s="23" t="inlineStr">
+        <is>
+          <t>3 пользователя. T-158/T-160 fixes работают</t>
+        </is>
+      </c>
+      <c r="H128" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I128" s="22" t="inlineStr">
+        <is>
+          <t>T-158</t>
+        </is>
+      </c>
+      <c r="J128" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="50" customHeight="1" s="15">
+      <c r="A129" s="22" t="inlineStr">
+        <is>
+          <t>TC-124</t>
+        </is>
+      </c>
+      <c r="B129" s="22" t="inlineStr">
+        <is>
+          <t>Timeline</t>
+        </is>
+      </c>
+      <c r="C129" s="23" t="inlineStr">
+        <is>
+          <t>Timeline - пользователи без focus data отображаются (T-160 fix)</t>
+        </is>
+      </c>
+      <c r="D129" s="23" t="inlineStr">
+        <is>
+          <t>Деплой с фиксом T-160 на test. Тенант имеет пользователей в device_user_sessions</t>
+        </is>
+      </c>
+      <c r="E129" s="22" t="inlineStr">
+        <is>
+          <t>1. Авторизоваться superadmin\n2. GET /users/timeline?date=2025-01-01&amp;timezone=Europe/Moscow&amp;tenant_id=...\n3. Проверить что API возвращает пользователей даже без focus intervals</t>
+        </is>
+      </c>
+      <c r="F129" s="22" t="inlineStr">
+        <is>
+          <t>Пользователи из device_user_sessions отображаются с пустыми hours</t>
+        </is>
+      </c>
+      <c r="G129" s="23" t="inlineStr">
+        <is>
+          <t>3 пользователя за прошлую дату с 0 hours</t>
+        </is>
+      </c>
+      <c r="H129" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I129" s="22" t="inlineStr">
+        <is>
+          <t>T-160</t>
+        </is>
+      </c>
+      <c r="J129" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="50" customHeight="1" s="15">
+      <c r="A130" s="22" t="inlineStr">
+        <is>
+          <t>TC-125</t>
+        </is>
+      </c>
+      <c r="B130" s="22" t="inlineStr">
+        <is>
+          <t>Timeline</t>
+        </is>
+      </c>
+      <c r="C130" s="23" t="inlineStr">
+        <is>
+          <t>Timeline - данные за сегодня</t>
+        </is>
+      </c>
+      <c r="D130" s="23" t="inlineStr">
+        <is>
+          <t>Деплой с фиксом T-158 на test</t>
+        </is>
+      </c>
+      <c r="E130" s="22" t="inlineStr">
+        <is>
+          <t>1. Авторизоваться superadmin\n2. GET /users/timeline?date=2026-03-10&amp;timezone=Europe/Moscow&amp;tenant_id=...\n3. Проверить данные за текущий день</t>
+        </is>
+      </c>
+      <c r="F130" s="22" t="inlineStr">
+        <is>
+          <t>Возвращаются пользователи с данными за сегодня (если были focus intervals)</t>
+        </is>
+      </c>
+      <c r="G130" s="23" t="inlineStr">
+        <is>
+          <t>3 пользователя за сегодня с 0 hours</t>
+        </is>
+      </c>
+      <c r="H130" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I130" s="22" t="inlineStr">
+        <is>
+          <t>T-158</t>
+        </is>
+      </c>
+      <c r="J130" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="50" customHeight="1" s="15">
+      <c r="A131" s="22" t="inlineStr">
+        <is>
+          <t>TC-126</t>
+        </is>
+      </c>
+      <c r="B131" s="22" t="inlineStr">
+        <is>
+          <t>Timeline</t>
+        </is>
+      </c>
+      <c r="C131" s="23" t="inlineStr">
+        <is>
+          <t>Timeline - невалидная дата возвращает 400 (T-156 recheck)</t>
+        </is>
+      </c>
+      <c r="D131" s="23" t="inlineStr">
+        <is>
+          <t>Деплой на test</t>
+        </is>
+      </c>
+      <c r="E131" s="22" t="inlineStr">
+        <is>
+          <t>1. Авторизоваться superadmin\n2. GET /users/timeline?date=invalid\n3. Проверить HTTP код</t>
+        </is>
+      </c>
+      <c r="F131" s="22" t="inlineStr">
+        <is>
+          <t>HTTP 400 Bad Request</t>
+        </is>
+      </c>
+      <c r="G131" s="23" t="inlineStr">
+        <is>
+          <t>HTTP 400 с Invalid date format</t>
+        </is>
+      </c>
+      <c r="H131" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I131" s="22" t="inlineStr">
+        <is>
+          <t>T-158</t>
+        </is>
+      </c>
+      <c r="J131" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="50" customHeight="1" s="15">
+      <c r="A132" s="22" t="inlineStr">
+        <is>
+          <t>TC-127</t>
+        </is>
+      </c>
+      <c r="B132" s="22" t="inlineStr">
+        <is>
+          <t>Timeline</t>
+        </is>
+      </c>
+      <c r="C132" s="23" t="inlineStr">
+        <is>
+          <t>Timeline - timezone UTC vs Moscow сдвигает часы на +3</t>
+        </is>
+      </c>
+      <c r="D132" s="23" t="inlineStr">
+        <is>
+          <t>Деплой с фиксом T-158 на test. Данные за 2026-03-09</t>
+        </is>
+      </c>
+      <c r="E132" s="22" t="inlineStr">
+        <is>
+          <t>1. Авторизоваться superadmin\n2. GET /users/timeline?date=2026-03-09&amp;timezone=UTC\n3. GET /users/timeline?date=2026-03-09&amp;timezone=Europe/Moscow\n4. Сравнить часы с данными</t>
+        </is>
+      </c>
+      <c r="F132" s="22" t="inlineStr">
+        <is>
+          <t>Часы в Moscow timezone сдвинуты на +3 относительно UTC</t>
+        </is>
+      </c>
+      <c r="G132" s="23" t="inlineStr">
+        <is>
+          <t>UTC hours +3 = Moscow hours верно</t>
+        </is>
+      </c>
+      <c r="H132" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I132" s="22" t="inlineStr">
+        <is>
+          <t>T-158</t>
+        </is>
+      </c>
+      <c r="J132" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="50" customHeight="1" s="15">
+      <c r="A133" s="22" t="inlineStr">
+        <is>
+          <t>TC-128</t>
+        </is>
+      </c>
+      <c r="B133" s="22" t="inlineStr">
+        <is>
+          <t>Catalogs</t>
+        </is>
+      </c>
+      <c r="C133" s="23" t="inlineStr">
+        <is>
+          <t>Catalogs groups - регрессия после timeline фикса</t>
+        </is>
+      </c>
+      <c r="D133" s="23" t="inlineStr">
+        <is>
+          <t>Деплой на test</t>
+        </is>
+      </c>
+      <c r="E133" s="22" t="inlineStr">
+        <is>
+          <t>1. Авторизоваться superadmin\n2. GET /catalogs/groups?group_type=APP&amp;tenant_id=...\n3. Проверить HTTP 200 и структуру ответа</t>
+        </is>
+      </c>
+      <c r="F133" s="22" t="inlineStr">
+        <is>
+          <t>HTTP 200, массив групп</t>
+        </is>
+      </c>
+      <c r="G133" s="23" t="inlineStr">
+        <is>
+          <t>HTTP 200, 9 APP групп</t>
+        </is>
+      </c>
+      <c r="H133" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I133" s="22" t="inlineStr">
+        <is>
+          <t>T-158</t>
+        </is>
+      </c>
+      <c r="J133" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="50" customHeight="1" s="15">
+      <c r="A134" s="22" t="inlineStr">
+        <is>
+          <t>TC-129</t>
+        </is>
+      </c>
+      <c r="B134" s="22" t="inlineStr">
+        <is>
+          <t>Web Dashboard</t>
+        </is>
+      </c>
+      <c r="C134" s="23" t="inlineStr">
+        <is>
+          <t>SPA загружается, favicon корректный</t>
+        </is>
+      </c>
+      <c r="D134" s="23" t="inlineStr">
+        <is>
+          <t>Деплой на test</t>
+        </is>
+      </c>
+      <c r="E134" s="22" t="inlineStr">
+        <is>
+          <t>1. GET /screenrecorder/\n2. Проверить HTTP 200\n3. Проверить favicon в HTML</t>
+        </is>
+      </c>
+      <c r="F134" s="22" t="inlineStr">
+        <is>
+          <t>HTTP 200, favicon присутствует</t>
+        </is>
+      </c>
+      <c r="G134" s="23" t="inlineStr">
+        <is>
+          <t>HTTP 200, favicon.png, title Кадеро</t>
+        </is>
+      </c>
+      <c r="H134" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I134" s="22" t="inlineStr">
+        <is>
+          <t>T-151</t>
+        </is>
+      </c>
+      <c r="J134" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="50" customHeight="1" s="15">
+      <c r="A135" s="22" t="inlineStr">
+        <is>
+          <t>TC-130</t>
+        </is>
+      </c>
+      <c r="B135" s="22" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C135" s="23" t="inlineStr">
+        <is>
+          <t>Dashboard group-timeline возвращает данные за период</t>
+        </is>
+      </c>
+      <c r="D135" s="23" t="inlineStr">
+        <is>
+          <t>Есть focus_intervals за 3+ дней</t>
+        </is>
+      </c>
+      <c r="E135" s="22" t="inlineStr">
+        <is>
+          <t>1. GET /dashboard/group-timeline?group_type=APP&amp;from=...&amp;to=...\n2. Проверить наличие groups, days, breakdown</t>
+        </is>
+      </c>
+      <c r="F135" s="22" t="inlineStr">
+        <is>
+          <t>groups содержит список групп с group_id/group_name/color. days содержит записи с breakdown, ungrouped_duration_ms, ungrouped_percentage</t>
+        </is>
+      </c>
+      <c r="G135" s="23" t="inlineStr">
+        <is>
+          <t>API возвращает 8 групп, 2 дня с breakdown, ungrouped_duration_ms=30004/1919997, ungrouped_percentage=0.23%/2.1%. Проценты рассчитаны корректно.</t>
+        </is>
+      </c>
+      <c r="H135" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I135" s="22" t="inlineStr">
+        <is>
+          <t>T-161</t>
+        </is>
+      </c>
+      <c r="J135" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="50" customHeight="1" s="15">
+      <c r="A136" s="22" t="inlineStr">
+        <is>
+          <t>TC-131</t>
+        </is>
+      </c>
+      <c r="B136" s="22" t="inlineStr">
+        <is>
+          <t>Timeline</t>
+        </is>
+      </c>
+      <c r="C136" s="23" t="inlineStr">
+        <is>
+          <t>Timeline has_recording корреляция с recording_sessions</t>
+        </is>
+      </c>
+      <c r="D136" s="23" t="inlineStr">
+        <is>
+          <t>Есть focus_intervals и recording_sessions за один день</t>
+        </is>
+      </c>
+      <c r="E136" s="22" t="inlineStr">
+        <is>
+          <t>1. GET /users/timeline?date=...\n2. Проверить has_recording для часов где есть сессии\n3. Проверить recording_session_ids</t>
+        </is>
+      </c>
+      <c r="F136" s="22" t="inlineStr">
+        <is>
+          <t>has_recording=true для часов с пересекающимися recording_sessions, recording_session_ids заполнены</t>
+        </is>
+      </c>
+      <c r="G136" s="23" t="inlineStr">
+        <is>
+          <t>has_recording=true для часов 0,10,11,12 (user AIR911D\ashep). recording_session_ids: 1,3,1,2 сессии. has_recording=false для часов 13,14 (нет записей).</t>
+        </is>
+      </c>
+      <c r="H136" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I136" s="22" t="inlineStr">
+        <is>
+          <t>T-162</t>
+        </is>
+      </c>
+      <c r="J136" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="50" customHeight="1" s="15">
+      <c r="A137" s="20" t="inlineStr">
+        <is>
+          <t>TC-132</t>
+        </is>
+      </c>
+      <c r="B137" s="20" t="inlineStr">
+        <is>
+          <t>Timeline</t>
+        </is>
+      </c>
+      <c r="C137" s="21" t="inlineStr">
+        <is>
+          <t>Timeline UI: видимые bars для групп и отдельных приложений</t>
+        </is>
+      </c>
+      <c r="D137" s="21" t="inlineStr">
+        <is>
+          <t>Есть focus_intervals с app_groups</t>
+        </is>
+      </c>
+      <c r="E137" s="20" t="inlineStr">
+        <is>
+          <t>1. Открыть страницу Аналитика &gt; Пользователи\n2. Развернуть пользователя\n3. Проверить наличие цветных баров для групп\n4. Развернуть группу — проверить бары для отдельных приложений</t>
+        </is>
+      </c>
+      <c r="F137" s="20" t="inlineStr">
+        <is>
+          <t>Группы отображаются цветными барами по часам. Отдельные приложения также отображают бары при раскрытии</t>
+        </is>
+      </c>
+      <c r="G137" s="21" t="inlineStr"/>
+      <c r="H137" s="20" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I137" s="20" t="inlineStr">
+        <is>
+          <t>T-163</t>
+        </is>
+      </c>
+      <c r="J137" s="21" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: employee groups, user activity, pipeline agents, docs, migrations
- Employee groups (CRUD, assign/unassign, sidebar, modal)
- User activity: recordings, worktime, apps/domains reports
- Employee list page with group filtering
- Auth: V30 token encryption, V35 employee permissions
- Ingest: V33 employee_groups tables, EmployeeGroupController
- Pipeline agents: architect, SA, BA, QA, UX/UI, BE, FE
- Docs: user-activity-tracking spec, macos-agent-parity, legal-saas,
  screen-action-analysis architecture, seed-test-data
- Nginx routes for ingest-gateway, k8s configmaps update

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracker.xlsx
+++ b/docs/tracker.xlsx
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I168"/>
+  <dimension ref="A1:I172"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="15" min="1" max="1"/>
@@ -8371,6 +8371,194 @@
         </is>
       </c>
     </row>
+    <row r="169" ht="20" customHeight="1" s="15">
+      <c r="A169" s="18" t="inlineStr">
+        <is>
+          <t>T-164</t>
+        </is>
+      </c>
+      <c r="B169" s="18" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C169" s="19" t="inlineStr">
+        <is>
+          <t>Справочники: вынести в отдельный пункт меню</t>
+        </is>
+      </c>
+      <c r="D169" s="19" t="inlineStr">
+        <is>
+          <t>Создать отдельный collapsible пункт основного меню Справочники между Аналитика и Настройки. Убрать Группы приложений и Группы сайтов из tenantSettingsSubmenu и superAdminSettingsSubmenu. Добавить isCatalogsExpanded state, isCatalogsActive, catalogsSubmenu. Файл: web-dashboard/src/components/Sidebar.tsx</t>
+        </is>
+      </c>
+      <c r="E169" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F169" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G169" s="19" t="inlineStr">
+        <is>
+          <t>Разработчик</t>
+        </is>
+      </c>
+      <c r="H169" s="18" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+      <c r="I169" s="18" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="20" customHeight="1" s="15">
+      <c r="A170" s="24" t="inlineStr">
+        <is>
+          <t>T-165</t>
+        </is>
+      </c>
+      <c r="B170" s="24" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C170" s="25" t="inlineStr">
+        <is>
+          <t>Tooltip дашборда: широкие строки и неверная сортировка групп</t>
+        </is>
+      </c>
+      <c r="D170" s="25" t="inlineStr">
+        <is>
+          <t>В GroupTimelineChart.tsx tooltip показывает группы в порядке sort_order (не по проценту) и с большим межстрочным интервалом. Нужен CustomTooltip компонент: сортировка payload по value desc + itemStyle padding 1px. Файл: web-dashboard/src/components/dashboard/GroupTimelineChart.tsx</t>
+        </is>
+      </c>
+      <c r="E170" s="24" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F170" s="24" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G170" s="25" t="inlineStr">
+        <is>
+          <t>Разработчик</t>
+        </is>
+      </c>
+      <c r="H170" s="24" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+      <c r="I170" s="24" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="20" customHeight="1" s="15">
+      <c r="A171" s="24" t="inlineStr">
+        <is>
+          <t>T-166</t>
+        </is>
+      </c>
+      <c r="B171" s="24" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C171" s="25" t="inlineStr">
+        <is>
+          <t>Timeline: группа Браузеры не показывает Группы сайтов</t>
+        </is>
+      </c>
+      <c r="D171" s="25" t="inlineStr">
+        <is>
+          <t>Корневая причина: в TimelineService группа Браузеры создаётся хардкодом с groupId=null и is_browser_group=true, но связи с конкретными APP-группами из БД нет. Если агент присылает browser-интервалы без домена (domain=null) — siteGroupMap пустой. Решение: добавить поле is_browser_group в app_groups (V32 миграция), использовать флаг из БД в TimelineService вместо хардкода. Затронутые файлы: V32__app_group_browser_flag.sql (новый), AppGroup.java, TimelineService.java, GroupCreateRequest.java, GroupUpdateRequest.java, GroupResponse.java, catalogs.ts, AppGroupsPage.tsx</t>
+        </is>
+      </c>
+      <c r="E171" s="24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F171" s="24" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G171" s="25" t="inlineStr">
+        <is>
+          <t>Разработчик</t>
+        </is>
+      </c>
+      <c r="H171" s="24" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+      <c r="I171" s="24" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="20" customHeight="1" s="15">
+      <c r="A172" s="18" t="inlineStr">
+        <is>
+          <t>T-167</t>
+        </is>
+      </c>
+      <c r="B172" s="18" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C172" s="19" t="inlineStr">
+        <is>
+          <t>recording_enabled toggle на device registration tokens</t>
+        </is>
+      </c>
+      <c r="D172" s="19" t="inlineStr">
+        <is>
+          <t>Фича: включение/отключение записи через toggle на registration token. V34 миграция, PATCH endpoint, каскад на device.settings, UI toggle, agent guards.</t>
+        </is>
+      </c>
+      <c r="E172" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F172" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G172" s="19" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="H172" s="18" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+      <c r="I172" s="18" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
@@ -8385,7 +8573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J137"/>
+  <dimension ref="A1:J149"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="15" min="1" max="1"/>
@@ -15324,6 +15512,630 @@
         </is>
       </c>
       <c r="J137" s="21" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="50" customHeight="1" s="15">
+      <c r="A138" s="22" t="inlineStr">
+        <is>
+          <t>TC-133</t>
+        </is>
+      </c>
+      <c r="B138" s="22" t="inlineStr">
+        <is>
+          <t>Device Tokens</t>
+        </is>
+      </c>
+      <c r="C138" s="23" t="inlineStr">
+        <is>
+          <t>POST token с recording_enabled=true</t>
+        </is>
+      </c>
+      <c r="D138" s="23" t="inlineStr">
+        <is>
+          <t>Авторизован как superadmin</t>
+        </is>
+      </c>
+      <c r="E138" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /api/v1/device-tokens с recording_enabled=true\n2. Проверить ответ</t>
+        </is>
+      </c>
+      <c r="F138" s="22" t="inlineStr">
+        <is>
+          <t>201, recording_enabled=true</t>
+        </is>
+      </c>
+      <c r="G138" s="23" t="inlineStr">
+        <is>
+          <t>Проверено после редеплоя 10.03.2026</t>
+        </is>
+      </c>
+      <c r="H138" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I138" s="22" t="inlineStr">
+        <is>
+          <t>T-167</t>
+        </is>
+      </c>
+      <c r="J138" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="50" customHeight="1" s="15">
+      <c r="A139" s="22" t="inlineStr">
+        <is>
+          <t>TC-134</t>
+        </is>
+      </c>
+      <c r="B139" s="22" t="inlineStr">
+        <is>
+          <t>Device Tokens</t>
+        </is>
+      </c>
+      <c r="C139" s="23" t="inlineStr">
+        <is>
+          <t>POST token с recording_enabled=false</t>
+        </is>
+      </c>
+      <c r="D139" s="23" t="inlineStr">
+        <is>
+          <t>Авторизован как superadmin</t>
+        </is>
+      </c>
+      <c r="E139" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /api/v1/device-tokens с recording_enabled=false\n2. Проверить ответ</t>
+        </is>
+      </c>
+      <c r="F139" s="22" t="inlineStr">
+        <is>
+          <t>201, recording_enabled=false</t>
+        </is>
+      </c>
+      <c r="G139" s="23" t="inlineStr">
+        <is>
+          <t>Проверено после редеплоя 10.03.2026</t>
+        </is>
+      </c>
+      <c r="H139" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I139" s="22" t="inlineStr">
+        <is>
+          <t>T-167</t>
+        </is>
+      </c>
+      <c r="J139" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="50" customHeight="1" s="15">
+      <c r="A140" s="22" t="inlineStr">
+        <is>
+          <t>TC-135</t>
+        </is>
+      </c>
+      <c r="B140" s="22" t="inlineStr">
+        <is>
+          <t>Device Tokens</t>
+        </is>
+      </c>
+      <c r="C140" s="23" t="inlineStr">
+        <is>
+          <t>POST token без recording_enabled (default=true)</t>
+        </is>
+      </c>
+      <c r="D140" s="23" t="inlineStr">
+        <is>
+          <t>Авторизован как superadmin</t>
+        </is>
+      </c>
+      <c r="E140" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /api/v1/device-tokens без recording_enabled\n2. Проверить ответ</t>
+        </is>
+      </c>
+      <c r="F140" s="22" t="inlineStr">
+        <is>
+          <t>201, recording_enabled=true (default)</t>
+        </is>
+      </c>
+      <c r="G140" s="23" t="inlineStr">
+        <is>
+          <t>Проверено после редеплоя 10.03.2026</t>
+        </is>
+      </c>
+      <c r="H140" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I140" s="22" t="inlineStr">
+        <is>
+          <t>T-167</t>
+        </is>
+      </c>
+      <c r="J140" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="50" customHeight="1" s="15">
+      <c r="A141" s="22" t="inlineStr">
+        <is>
+          <t>TC-136</t>
+        </is>
+      </c>
+      <c r="B141" s="22" t="inlineStr">
+        <is>
+          <t>Device Tokens</t>
+        </is>
+      </c>
+      <c r="C141" s="23" t="inlineStr">
+        <is>
+          <t>PATCH recording_enabled=false</t>
+        </is>
+      </c>
+      <c r="D141" s="23" t="inlineStr">
+        <is>
+          <t>Авторизован как superadmin, токен существует</t>
+        </is>
+      </c>
+      <c r="E141" s="22" t="inlineStr">
+        <is>
+          <t>1. PATCH /api/v1/device-tokens/{id} с recording_enabled=false\n2. Проверить ответ</t>
+        </is>
+      </c>
+      <c r="F141" s="22" t="inlineStr">
+        <is>
+          <t>200, recording_enabled=false</t>
+        </is>
+      </c>
+      <c r="G141" s="23" t="inlineStr">
+        <is>
+          <t>Проверено после редеплоя 10.03.2026</t>
+        </is>
+      </c>
+      <c r="H141" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I141" s="22" t="inlineStr">
+        <is>
+          <t>T-167</t>
+        </is>
+      </c>
+      <c r="J141" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="50" customHeight="1" s="15">
+      <c r="A142" s="22" t="inlineStr">
+        <is>
+          <t>TC-137</t>
+        </is>
+      </c>
+      <c r="B142" s="22" t="inlineStr">
+        <is>
+          <t>Device Tokens</t>
+        </is>
+      </c>
+      <c r="C142" s="23" t="inlineStr">
+        <is>
+          <t>PATCH recording_enabled=true</t>
+        </is>
+      </c>
+      <c r="D142" s="23" t="inlineStr">
+        <is>
+          <t>Авторизован как superadmin, токен с recording_enabled=false</t>
+        </is>
+      </c>
+      <c r="E142" s="22" t="inlineStr">
+        <is>
+          <t>1. PATCH /api/v1/device-tokens/{id} с recording_enabled=true\n2. Проверить ответ</t>
+        </is>
+      </c>
+      <c r="F142" s="22" t="inlineStr">
+        <is>
+          <t>200, recording_enabled=true</t>
+        </is>
+      </c>
+      <c r="G142" s="23" t="inlineStr">
+        <is>
+          <t>Проверено после редеплоя 10.03.2026</t>
+        </is>
+      </c>
+      <c r="H142" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I142" s="22" t="inlineStr">
+        <is>
+          <t>T-167</t>
+        </is>
+      </c>
+      <c r="J142" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="50" customHeight="1" s="15">
+      <c r="A143" s="22" t="inlineStr">
+        <is>
+          <t>TC-138</t>
+        </is>
+      </c>
+      <c r="B143" s="22" t="inlineStr">
+        <is>
+          <t>Device Tokens</t>
+        </is>
+      </c>
+      <c r="C143" s="23" t="inlineStr">
+        <is>
+          <t>PATCH name на token</t>
+        </is>
+      </c>
+      <c r="D143" s="23" t="inlineStr">
+        <is>
+          <t>Авторизован как superadmin, токен существует</t>
+        </is>
+      </c>
+      <c r="E143" s="22" t="inlineStr">
+        <is>
+          <t>1. PATCH /api/v1/device-tokens/{id} с name=new-name\n2. Проверить ответ</t>
+        </is>
+      </c>
+      <c r="F143" s="22" t="inlineStr">
+        <is>
+          <t>200, name обновлено</t>
+        </is>
+      </c>
+      <c r="G143" s="23" t="inlineStr">
+        <is>
+          <t>Проверено после редеплоя 10.03.2026</t>
+        </is>
+      </c>
+      <c r="H143" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I143" s="22" t="inlineStr">
+        <is>
+          <t>T-167</t>
+        </is>
+      </c>
+      <c r="J143" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="50" customHeight="1" s="15">
+      <c r="A144" s="22" t="inlineStr">
+        <is>
+          <t>TC-139</t>
+        </is>
+      </c>
+      <c r="B144" s="22" t="inlineStr">
+        <is>
+          <t>Device Tokens</t>
+        </is>
+      </c>
+      <c r="C144" s="23" t="inlineStr">
+        <is>
+          <t>PATCH max_uses на token</t>
+        </is>
+      </c>
+      <c r="D144" s="23" t="inlineStr">
+        <is>
+          <t>Авторизован как superadmin, токен существует</t>
+        </is>
+      </c>
+      <c r="E144" s="22" t="inlineStr">
+        <is>
+          <t>1. PATCH /api/v1/device-tokens/{id} с max_uses=99\n2. Проверить ответ</t>
+        </is>
+      </c>
+      <c r="F144" s="22" t="inlineStr">
+        <is>
+          <t>200, max_uses=99</t>
+        </is>
+      </c>
+      <c r="G144" s="23" t="inlineStr">
+        <is>
+          <t>Проверено после редеплоя 10.03.2026</t>
+        </is>
+      </c>
+      <c r="H144" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I144" s="22" t="inlineStr">
+        <is>
+          <t>T-167</t>
+        </is>
+      </c>
+      <c r="J144" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="50" customHeight="1" s="15">
+      <c r="A145" s="22" t="inlineStr">
+        <is>
+          <t>TC-140</t>
+        </is>
+      </c>
+      <c r="B145" s="22" t="inlineStr">
+        <is>
+          <t>Device Tokens</t>
+        </is>
+      </c>
+      <c r="C145" s="23" t="inlineStr">
+        <is>
+          <t>PATCH cross-tenant isolation</t>
+        </is>
+      </c>
+      <c r="D145" s="23" t="inlineStr">
+        <is>
+          <t>Авторизован как test user (tenant test-org)</t>
+        </is>
+      </c>
+      <c r="E145" s="22" t="inlineStr">
+        <is>
+          <t>1. PATCH /api/v1/device-tokens/{id} токена из другого тенанта\n2. Проверить ответ</t>
+        </is>
+      </c>
+      <c r="F145" s="22" t="inlineStr">
+        <is>
+          <t>404 (tenant isolation)</t>
+        </is>
+      </c>
+      <c r="G145" s="23" t="inlineStr">
+        <is>
+          <t>Проверено после редеплоя 10.03.2026</t>
+        </is>
+      </c>
+      <c r="H145" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I145" s="22" t="inlineStr">
+        <is>
+          <t>T-167</t>
+        </is>
+      </c>
+      <c r="J145" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="50" customHeight="1" s="15">
+      <c r="A146" s="22" t="inlineStr">
+        <is>
+          <t>TC-141</t>
+        </is>
+      </c>
+      <c r="B146" s="22" t="inlineStr">
+        <is>
+          <t>Device Tokens</t>
+        </is>
+      </c>
+      <c r="C146" s="23" t="inlineStr">
+        <is>
+          <t>PATCH несуществующий токен</t>
+        </is>
+      </c>
+      <c r="D146" s="23" t="inlineStr">
+        <is>
+          <t>Авторизован как superadmin</t>
+        </is>
+      </c>
+      <c r="E146" s="22" t="inlineStr">
+        <is>
+          <t>1. PATCH /api/v1/device-tokens/{random-uuid}\n2. Проверить ответ</t>
+        </is>
+      </c>
+      <c r="F146" s="22" t="inlineStr">
+        <is>
+          <t>404 Not Found</t>
+        </is>
+      </c>
+      <c r="G146" s="23" t="inlineStr">
+        <is>
+          <t>Проверено после редеплоя 10.03.2026</t>
+        </is>
+      </c>
+      <c r="H146" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I146" s="22" t="inlineStr">
+        <is>
+          <t>T-167</t>
+        </is>
+      </c>
+      <c r="J146" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="50" customHeight="1" s="15">
+      <c r="A147" s="22" t="inlineStr">
+        <is>
+          <t>TC-142</t>
+        </is>
+      </c>
+      <c r="B147" s="22" t="inlineStr">
+        <is>
+          <t>Device Tokens</t>
+        </is>
+      </c>
+      <c r="C147" s="23" t="inlineStr">
+        <is>
+          <t>Device-login server_config содержит recording_enabled</t>
+        </is>
+      </c>
+      <c r="D147" s="23" t="inlineStr">
+        <is>
+          <t>Registration token существует, активен</t>
+        </is>
+      </c>
+      <c r="E147" s="22" t="inlineStr">
+        <is>
+          <t>1. POST /api/v1/auth/device-login\n2. Проверить server_config</t>
+        </is>
+      </c>
+      <c r="F147" s="22" t="inlineStr">
+        <is>
+          <t>server_config.recording_enabled=true/false</t>
+        </is>
+      </c>
+      <c r="G147" s="23" t="inlineStr">
+        <is>
+          <t>Проверено после редеплоя 10.03.2026</t>
+        </is>
+      </c>
+      <c r="H147" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I147" s="22" t="inlineStr">
+        <is>
+          <t>T-167</t>
+        </is>
+      </c>
+      <c r="J147" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="50" customHeight="1" s="15">
+      <c r="A148" s="22" t="inlineStr">
+        <is>
+          <t>TC-143</t>
+        </is>
+      </c>
+      <c r="B148" s="22" t="inlineStr">
+        <is>
+          <t>Device Tokens</t>
+        </is>
+      </c>
+      <c r="C148" s="23" t="inlineStr">
+        <is>
+          <t>Audit log при PATCH recording_enabled</t>
+        </is>
+      </c>
+      <c r="D148" s="23" t="inlineStr">
+        <is>
+          <t>Авторизован как superadmin</t>
+        </is>
+      </c>
+      <c r="E148" s="22" t="inlineStr">
+        <is>
+          <t>1. PATCH recording_enabled\n2. Проверить audit log в БД</t>
+        </is>
+      </c>
+      <c r="F148" s="22" t="inlineStr">
+        <is>
+          <t>action=DEVICE_TOKEN_UPDATED записано</t>
+        </is>
+      </c>
+      <c r="G148" s="23" t="inlineStr">
+        <is>
+          <t>Проверено после редеплоя 10.03.2026</t>
+        </is>
+      </c>
+      <c r="H148" s="22" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I148" s="22" t="inlineStr">
+        <is>
+          <t>T-167</t>
+        </is>
+      </c>
+      <c r="J148" s="23" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="50" customHeight="1" s="15">
+      <c r="A149" s="20" t="inlineStr">
+        <is>
+          <t>TC-144</t>
+        </is>
+      </c>
+      <c r="B149" s="20" t="inlineStr">
+        <is>
+          <t>Device Tokens</t>
+        </is>
+      </c>
+      <c r="C149" s="21" t="inlineStr">
+        <is>
+          <t>UI toggle recording_enabled в списке токенов</t>
+        </is>
+      </c>
+      <c r="D149" s="21" t="inlineStr">
+        <is>
+          <t>Авторизован в web-dashboard</t>
+        </is>
+      </c>
+      <c r="E149" s="20" t="inlineStr">
+        <is>
+          <t>1. Открыть Настройки → Токены\n2. Переключить toggle Запись\n3. Обновить страницу</t>
+        </is>
+      </c>
+      <c r="F149" s="20" t="inlineStr">
+        <is>
+          <t>Toggle переключается, значение сохраняется</t>
+        </is>
+      </c>
+      <c r="G149" s="21" t="inlineStr">
+        <is>
+          <t>Ожидает ручной проверки в UI</t>
+        </is>
+      </c>
+      <c r="H149" s="20" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="I149" s="20" t="inlineStr">
+        <is>
+          <t>T-167</t>
+        </is>
+      </c>
+      <c r="J149" s="21" t="inlineStr">
         <is>
           <t>10.03.2026</t>
         </is>

</xml_diff>

<commit_message>
docs: T-175 username uniqueness analysis + decomposition into 7 subtasks
- T-175 analysis: global unique username (= email), registration flow,
  duplicate handling, SMTP config, tenant memberships
- Decomposed into 7 subtasks (T-175.1 through T-175.7) with 64 test cases
- Phase A: DB migration + backend uniqueness + login + frontend
- Phase B: tenant_memberships architecture
- Phase C: SMTP + email invitations
- Updated agent-upload-redesign checklist (14/17 PASS)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracker.xlsx
+++ b/docs/tracker.xlsx
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I179"/>
+  <dimension ref="A1:I180"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="15" min="1" max="1"/>
@@ -8976,6 +8976,53 @@
         </is>
       </c>
     </row>
+    <row r="180" ht="20" customHeight="1" s="15">
+      <c r="A180" s="24" t="inlineStr">
+        <is>
+          <t>T-175</t>
+        </is>
+      </c>
+      <c r="B180" s="24" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="C180" s="25" t="inlineStr">
+        <is>
+          <t>Нет глобальной проверки уникальности username — конфликт при логине</t>
+        </is>
+      </c>
+      <c r="D180" s="25" t="inlineStr">
+        <is>
+          <t>Username уникален только в рамках тенанта. При логине без slug — если два пользователя с одинаковым username в разных тенантах, система берёт первого. Второй не может залогиниться. Race condition при создании → 500 вместо 409. Аналитика: docs/ToDo/T-175-уникальность-username-при-регистрации.md</t>
+        </is>
+      </c>
+      <c r="E180" s="24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F180" s="24" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G180" s="25" t="inlineStr">
+        <is>
+          <t>Разработчик</t>
+        </is>
+      </c>
+      <c r="H180" s="24" t="inlineStr">
+        <is>
+          <t>20.03.2026</t>
+        </is>
+      </c>
+      <c r="I180" s="24" t="inlineStr">
+        <is>
+          <t>20.03.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
feat(T-176): @Scheduled device timeout — auto-offline after 90s without heartbeat
- DeviceTimeoutService: @Scheduled(60s) checks last_heartbeat_ts
- Devices with no heartbeat for >90s → status = "offline"
- Native INSERT into device_status_log (bypass immutable UPDATE trigger)
- DeviceRepository.findStaleDevices() query
- ControlPlaneApplication: @EnableScheduling
- Configurable: prg.device-timeout.stale-threshold-sec, check-interval-ms

Tested: 15/16 stale devices marked offline, DESKTOP-J15ON4Q recording→offline,
device_status_log entries with trigger="system"

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracker.xlsx
+++ b/docs/tracker.xlsx
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I180"/>
+  <dimension ref="A1:I181"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="15" min="1" max="1"/>
@@ -9023,6 +9023,53 @@
         </is>
       </c>
     </row>
+    <row r="181" ht="20" customHeight="1" s="15">
+      <c r="A181" s="18" t="inlineStr">
+        <is>
+          <t>T-176</t>
+        </is>
+      </c>
+      <c r="B181" s="18" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C181" s="19" t="inlineStr">
+        <is>
+          <t>Серверный таймаут устройств: @Scheduled перевод в offline при отсутствии heartbeat</t>
+        </is>
+      </c>
+      <c r="D181" s="19" t="inlineStr">
+        <is>
+          <t>Control-plane @Scheduled(60s): если last_heartbeat_ts &gt; 90с → status=offline. Записывать в device_status_log. Аналитика: docs/ToDo/T-176-серверный-таймаут-устройств.md</t>
+        </is>
+      </c>
+      <c r="E181" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F181" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G181" s="19" t="inlineStr">
+        <is>
+          <t>Разработчик</t>
+        </is>
+      </c>
+      <c r="H181" s="18" t="inlineStr">
+        <is>
+          <t>20.03.2026</t>
+        </is>
+      </c>
+      <c r="I181" s="18" t="inlineStr">
+        <is>
+          <t>20.03.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
docs: T-177 mobile adaptation — decomposition into 9 subtasks
- 00-overview: порядок реализации, тестовые устройства
- 01: SessionDetailPage grid-cols-3 (critical)
- 02: UserReportsPage tab-nav overflow
- 03: TimelinesPage date picker + filters
- 04: DeviceTokensList hidden columns
- 05: EmployeeList sidebar → collapsible
- 06: DevicesList sidebar → collapsible
- 07: SearchPage filters column layout
- 08: Bulk table column hiding (5 tables)
- 09: Forms + widgets touch target check

T-176 device timeout task file

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracker.xlsx
+++ b/docs/tracker.xlsx
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I181"/>
+  <dimension ref="A1:I182"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="15" min="1" max="1"/>
@@ -9070,6 +9070,53 @@
         </is>
       </c>
     </row>
+    <row r="182" ht="20" customHeight="1" s="15">
+      <c r="A182" s="18" t="inlineStr">
+        <is>
+          <t>T-177</t>
+        </is>
+      </c>
+      <c r="B182" s="18" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C182" s="19" t="inlineStr">
+        <is>
+          <t>Мобильная адаптация web-dashboard: 16 подзадач по страницам</t>
+        </is>
+      </c>
+      <c r="D182" s="19" t="inlineStr">
+        <is>
+          <t>Адаптация всех 38 страниц к мобильным устройствам (320-428px). 1 critical (SessionDetailPage grid-cols-3), 5 high, 5 medium, 5 low. Аналитика: docs/ToDo/T-177-мобильная-адаптация-веба.md</t>
+        </is>
+      </c>
+      <c r="E182" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F182" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G182" s="19" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+      <c r="H182" s="18" t="inlineStr">
+        <is>
+          <t>20.03.2026</t>
+        </is>
+      </c>
+      <c r="I182" s="18" t="inlineStr">
+        <is>
+          <t>20.03.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
docs: T-178 production deployment kadero.online (2 app servers + 1 LB)
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracker.xlsx
+++ b/docs/tracker.xlsx
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I182"/>
+  <dimension ref="A1:I183"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="15" min="1" max="1"/>
@@ -9117,6 +9117,53 @@
         </is>
       </c>
     </row>
+    <row r="183" ht="20" customHeight="1" s="15">
+      <c r="A183" s="18" t="inlineStr">
+        <is>
+          <t>T-178</t>
+        </is>
+      </c>
+      <c r="B183" s="18" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C183" s="19" t="inlineStr">
+        <is>
+          <t>Развёртывание промышленного контура kadero.online (2 app + 1 LB)</t>
+        </is>
+      </c>
+      <c r="D183" s="19" t="inlineStr">
+        <is>
+          <t>3 сервера: 2×(8vCPU/16GB/150GB) app + 1 LB. PostgreSQL primary+replica, MinIO distributed, Kafka 2 brokers, OpenSearch 2 nodes. nginx LB + SSL. Аналитика: docs/ToDo/T-178-промышленный-контур-kadero-online.md</t>
+        </is>
+      </c>
+      <c r="E183" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F183" s="18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G183" s="19" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="H183" s="18" t="inlineStr">
+        <is>
+          <t>20.03.2026</t>
+        </is>
+      </c>
+      <c r="I183" s="18" t="inlineStr">
+        <is>
+          <t>20.03.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
feat(auth): T-179 switch SMTP to noreply@shepaland.ru via STARTTLS 587
- Switch from otp@shepaland.ru (SSL/465) to noreply@shepaland.ru (STARTTLS/587)
- Fix findActiveByEmail: LEFT JOIN FETCH roles/permissions (invited users without direct roles were not found on auto-login)
- Add SMTP config to prod configmaps/secrets
- Update NetworkPolicy: port 465 → 587

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracker.xlsx
+++ b/docs/tracker.xlsx
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I183"/>
+  <dimension ref="A1:I184"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="15" min="1" max="1"/>
@@ -9164,6 +9164,53 @@
         </is>
       </c>
     </row>
+    <row r="184" ht="20" customHeight="1" s="15">
+      <c r="A184" s="18" t="inlineStr">
+        <is>
+          <t>T-179</t>
+        </is>
+      </c>
+      <c r="B184" s="18" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C184" s="19" t="inlineStr">
+        <is>
+          <t>Настройка отправки почты: noreply@shepaland.ru через reg.ru SMTP</t>
+        </is>
+      </c>
+      <c r="D184" s="19" t="inlineStr">
+        <is>
+          <t>Переключить email-отправку с otp@shepaland.ru на noreply@shepaland.ru. Обновить конфигурацию на test и prod. Решить проблему блокировки SMTP на Yandex Cloud (test). Аналитика: docs/todo/T-179-настройка-отправки-почты.md</t>
+        </is>
+      </c>
+      <c r="E184" s="18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F184" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G184" s="19" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="H184" s="18" t="inlineStr">
+        <is>
+          <t>22.03.2026</t>
+        </is>
+      </c>
+      <c r="I184" s="18" t="inlineStr">
+        <is>
+          <t>22.03.2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>